<commit_message>
Save pending crossword question bank edits
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -4843,149 +4843,601 @@
       </c>
     </row>
     <row r="218" ht="21.95" customHeight="1">
-      <c r="C218" s="2" t="n"/>
-      <c r="D218" s="2" t="n"/>
-      <c r="E218" s="2" t="n"/>
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Organ whose regions
+  form networks</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>BRAIN</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr"/>
+      <c r="D218" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E218" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="219" ht="21.95" customHeight="1">
-      <c r="C219" s="2" t="n"/>
-      <c r="D219" s="2" t="n"/>
-      <c r="E219" s="2" t="n"/>
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Where interoception gets its signals</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>BODY</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr"/>
+      <c r="D219" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E219" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="220" ht="21.95" customHeight="1">
-      <c r="C220" s="2" t="n"/>
-      <c r="D220" s="2" t="n"/>
-      <c r="E220" s="2" t="n"/>
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Brain areas don't work solo; they're a...</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr"/>
+      <c r="D220" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E220" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="221" ht="21.95" customHeight="1">
-      <c r="C221" s="2" t="n"/>
-      <c r="D221" s="2" t="n"/>
-      <c r="E221" s="2" t="n"/>
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>What a weak leg may struggle to do</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>MOVE</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr"/>
+      <c r="D221" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E221" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="222" ht="21.95" customHeight="1">
-      <c r="C222" s="2" t="n"/>
-      <c r="D222" s="2" t="n"/>
-      <c r="E222" s="2" t="n"/>
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Changing this may change a movement</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>TASK</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr"/>
+      <c r="D222" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E222" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="223" ht="21.95" customHeight="1">
-      <c r="C223" s="2" t="n"/>
-      <c r="D223" s="2" t="n"/>
-      <c r="E223" s="2" t="n"/>
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>To direct attention toward one thing</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>FOCUS</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr"/>
+      <c r="D223" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E223" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="224" ht="21.95" customHeight="1">
-      <c r="C224" s="2" t="n"/>
-      <c r="D224" s="2" t="n"/>
-      <c r="E224" s="2" t="n"/>
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>A loud one can steal the spotlight</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>NOISE</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr"/>
+      <c r="D224" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E224" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="225" ht="21.95" customHeight="1">
-      <c r="C225" s="2" t="n"/>
-      <c r="D225" s="2" t="n"/>
-      <c r="E225" s="2" t="n"/>
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Unwelcome body signal that grabs
+  attention</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>PAIN</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr"/>
+      <c r="D225" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E225" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="226" ht="21.95" customHeight="1">
-      <c r="C226" s="2" t="n"/>
-      <c r="D226" s="2" t="n"/>
-      <c r="E226" s="2" t="n"/>
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>May accompany functional seizures or
+  panic</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>FEAR</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr"/>
+      <c r="D226" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E226" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="227" ht="21.95" customHeight="1">
-      <c r="C227" s="2" t="n"/>
-      <c r="D227" s="2" t="n"/>
-      <c r="E227" s="2" t="n"/>
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Attack often involving sudden intense
+  fear</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>PANIC</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr"/>
+      <c r="D227" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E227" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="228" ht="21.95" customHeight="1">
-      <c r="C228" s="2" t="n"/>
-      <c r="D228" s="2" t="n"/>
-      <c r="E228" s="2" t="n"/>
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Three-letter scan used to study brain
+  structure</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>MRI</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr"/>
+      <c r="D228" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E228" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="229" ht="21.95" customHeight="1">
-      <c r="C229" s="2" t="n"/>
-      <c r="D229" s="2" t="n"/>
-      <c r="E229" s="2" t="n"/>
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Examination finding supporting an FND
+  diagnosis</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>SIGN</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr"/>
+      <c r="D229" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E229" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="230" ht="21.95" customHeight="1">
-      <c r="C230" s="2" t="n"/>
-      <c r="D230" s="2" t="n"/>
-      <c r="E230" s="2" t="n"/>
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>A break that may help manage daily
+  demands</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr"/>
+      <c r="D230" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E230" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="231" ht="21.95" customHeight="1">
-      <c r="C231" s="2" t="n"/>
-      <c r="D231" s="2" t="n"/>
-      <c r="E231" s="2" t="n"/>
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>The brain borrows experience from here</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>PAST</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr"/>
+      <c r="D231" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E231" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="232" ht="21.95" customHeight="1">
-      <c r="C232" s="2" t="n"/>
-      <c r="D232" s="2" t="n"/>
-      <c r="E232" s="2" t="n"/>
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Its beat provides internal body signals</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>HEART</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr"/>
+      <c r="D232" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E232" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="233" ht="21.95" customHeight="1">
-      <c r="C233" s="2" t="n"/>
-      <c r="D233" s="2" t="n"/>
-      <c r="E233" s="2" t="n"/>
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Team of brain areas sharing information</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>NETWORK</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E233" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="234" ht="21.95" customHeight="1">
-      <c r="C234" s="2" t="n"/>
-      <c r="D234" s="2" t="n"/>
-      <c r="E234" s="2" t="n"/>
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Sense of making an action happen</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E234" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="235" ht="21.95" customHeight="1">
-      <c r="C235" s="2" t="n"/>
-      <c r="D235" s="2" t="n"/>
-      <c r="E235" s="2" t="n"/>
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Shaking that may change during another
+  task</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>TREMOR</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr"/>
+      <c r="D235" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E235" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="236" ht="21.95" customHeight="1">
-      <c r="C236" s="2" t="n"/>
-      <c r="D236" s="2" t="n"/>
-      <c r="E236" s="2" t="n"/>
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Pattern of beats examined in tremor</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>RHYTHM</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr"/>
+      <c r="D236" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E236" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="237" ht="21.95" customHeight="1">
-      <c r="C237" s="2" t="n"/>
-      <c r="D237" s="2" t="n"/>
-      <c r="E237" s="2" t="n"/>
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Message sent between the body and brain</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E237" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="238" ht="21.95" customHeight="1">
-      <c r="C238" s="2" t="n"/>
-      <c r="D238" s="2" t="n"/>
-      <c r="E238" s="2" t="n"/>
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Brain ability that may slip out of reach</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>MEMORY</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E238" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="239" ht="21.95" customHeight="1">
-      <c r="C239" s="2" t="n"/>
-      <c r="D239" s="2" t="n"/>
-      <c r="E239" s="2" t="n"/>
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Describes evidence gathered by the senses</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>SENSORY</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E239" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="240" ht="21.95" customHeight="1">
-      <c r="C240" s="2" t="n"/>
-      <c r="D240" s="2" t="n"/>
-      <c r="E240" s="2" t="n"/>
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Functional event involving altered
+  awareness or movement</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>SEIZURE</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr"/>
+      <c r="D240" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E240" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="241" ht="21.95" customHeight="1">
-      <c r="C241" s="2" t="n"/>
-      <c r="D241" s="2" t="n"/>
-      <c r="E241" s="2" t="n"/>
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Movement can involve automatic or focused
+  forms of this</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E241" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="242" ht="21.95" customHeight="1">
-      <c r="C242" s="2" t="n"/>
-      <c r="D242" s="2" t="n"/>
-      <c r="E242" s="2" t="n"/>
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Messenger used alongside electrical
+  activity</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>CHEMICAL</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E242" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="243" ht="21.95" customHeight="1">
-      <c r="C243" s="2" t="n"/>
-      <c r="D243" s="2" t="n"/>
-      <c r="E243" s="2" t="n"/>
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Brain's spotlight, sometimes stolen by
+  noise</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>ATTENTION</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr"/>
+      <c r="D243" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E243" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="244" ht="21.95" customHeight="1">
-      <c r="C244" s="2" t="n"/>
-      <c r="D244" s="2" t="n"/>
-      <c r="E244" s="2" t="n"/>
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Brain's best guess about what's coming</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>PREDICTION</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E244" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="245" ht="21.95" customHeight="1">
-      <c r="C245" s="2" t="n"/>
-      <c r="D245" s="2" t="n"/>
-      <c r="E245" s="2" t="n"/>
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Movement control without step-by-step
+  planning</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>AUTOMATIC</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr"/>
+      <c r="D245" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E245" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="246" ht="21.95" customHeight="1">
-      <c r="C246" s="2" t="n"/>
-      <c r="D246" s="2" t="n"/>
-      <c r="E246" s="2" t="n"/>
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Sensing and interpreting signals inside
+  the body</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>INTEROCEPTION</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr"/>
+      <c r="D246" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E246" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="247" ht="21.95" customHeight="1">
       <c r="C247" s="2" t="n"/>

</xml_diff>

<commit_message>
Save pending crossword question-bank edits (#169)
## Purpose
Preserve the edited Excel crossword question bank from the Codespace
before starting a new workshop session.

## Scope
- Only `tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx` is
changed.
- No public course pages, published puzzles, code, or site assets are
modified.

## Next step
Review the workbook, merge this PR into `main`, and then update the
Codespace's local `main` branch. Clear the local Wrangler cache only
after checking Git status. This PR does not clean up local untracked
files.
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -4843,149 +4843,601 @@
       </c>
     </row>
     <row r="218" ht="21.95" customHeight="1">
-      <c r="C218" s="2" t="n"/>
-      <c r="D218" s="2" t="n"/>
-      <c r="E218" s="2" t="n"/>
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Organ whose regions
+  form networks</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>BRAIN</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr"/>
+      <c r="D218" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E218" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="219" ht="21.95" customHeight="1">
-      <c r="C219" s="2" t="n"/>
-      <c r="D219" s="2" t="n"/>
-      <c r="E219" s="2" t="n"/>
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Where interoception gets its signals</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>BODY</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr"/>
+      <c r="D219" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E219" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="220" ht="21.95" customHeight="1">
-      <c r="C220" s="2" t="n"/>
-      <c r="D220" s="2" t="n"/>
-      <c r="E220" s="2" t="n"/>
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Brain areas don't work solo; they're a...</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr"/>
+      <c r="D220" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E220" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="221" ht="21.95" customHeight="1">
-      <c r="C221" s="2" t="n"/>
-      <c r="D221" s="2" t="n"/>
-      <c r="E221" s="2" t="n"/>
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>What a weak leg may struggle to do</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>MOVE</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr"/>
+      <c r="D221" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E221" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="222" ht="21.95" customHeight="1">
-      <c r="C222" s="2" t="n"/>
-      <c r="D222" s="2" t="n"/>
-      <c r="E222" s="2" t="n"/>
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Changing this may change a movement</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>TASK</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr"/>
+      <c r="D222" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E222" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="223" ht="21.95" customHeight="1">
-      <c r="C223" s="2" t="n"/>
-      <c r="D223" s="2" t="n"/>
-      <c r="E223" s="2" t="n"/>
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>To direct attention toward one thing</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>FOCUS</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr"/>
+      <c r="D223" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E223" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="224" ht="21.95" customHeight="1">
-      <c r="C224" s="2" t="n"/>
-      <c r="D224" s="2" t="n"/>
-      <c r="E224" s="2" t="n"/>
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>A loud one can steal the spotlight</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>NOISE</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr"/>
+      <c r="D224" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E224" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="225" ht="21.95" customHeight="1">
-      <c r="C225" s="2" t="n"/>
-      <c r="D225" s="2" t="n"/>
-      <c r="E225" s="2" t="n"/>
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Unwelcome body signal that grabs
+  attention</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>PAIN</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr"/>
+      <c r="D225" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E225" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="226" ht="21.95" customHeight="1">
-      <c r="C226" s="2" t="n"/>
-      <c r="D226" s="2" t="n"/>
-      <c r="E226" s="2" t="n"/>
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>May accompany functional seizures or
+  panic</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>FEAR</t>
+        </is>
+      </c>
+      <c r="C226" s="2" t="inlineStr"/>
+      <c r="D226" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E226" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="227" ht="21.95" customHeight="1">
-      <c r="C227" s="2" t="n"/>
-      <c r="D227" s="2" t="n"/>
-      <c r="E227" s="2" t="n"/>
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Attack often involving sudden intense
+  fear</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>PANIC</t>
+        </is>
+      </c>
+      <c r="C227" s="2" t="inlineStr"/>
+      <c r="D227" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E227" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="228" ht="21.95" customHeight="1">
-      <c r="C228" s="2" t="n"/>
-      <c r="D228" s="2" t="n"/>
-      <c r="E228" s="2" t="n"/>
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Three-letter scan used to study brain
+  structure</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>MRI</t>
+        </is>
+      </c>
+      <c r="C228" s="2" t="inlineStr"/>
+      <c r="D228" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E228" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="229" ht="21.95" customHeight="1">
-      <c r="C229" s="2" t="n"/>
-      <c r="D229" s="2" t="n"/>
-      <c r="E229" s="2" t="n"/>
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Examination finding supporting an FND
+  diagnosis</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>SIGN</t>
+        </is>
+      </c>
+      <c r="C229" s="2" t="inlineStr"/>
+      <c r="D229" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E229" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="230" ht="21.95" customHeight="1">
-      <c r="C230" s="2" t="n"/>
-      <c r="D230" s="2" t="n"/>
-      <c r="E230" s="2" t="n"/>
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>A break that may help manage daily
+  demands</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="C230" s="2" t="inlineStr"/>
+      <c r="D230" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E230" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="231" ht="21.95" customHeight="1">
-      <c r="C231" s="2" t="n"/>
-      <c r="D231" s="2" t="n"/>
-      <c r="E231" s="2" t="n"/>
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>The brain borrows experience from here</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>PAST</t>
+        </is>
+      </c>
+      <c r="C231" s="2" t="inlineStr"/>
+      <c r="D231" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E231" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="232" ht="21.95" customHeight="1">
-      <c r="C232" s="2" t="n"/>
-      <c r="D232" s="2" t="n"/>
-      <c r="E232" s="2" t="n"/>
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Its beat provides internal body signals</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>HEART</t>
+        </is>
+      </c>
+      <c r="C232" s="2" t="inlineStr"/>
+      <c r="D232" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E232" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="233" ht="21.95" customHeight="1">
-      <c r="C233" s="2" t="n"/>
-      <c r="D233" s="2" t="n"/>
-      <c r="E233" s="2" t="n"/>
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Team of brain areas sharing information</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>NETWORK</t>
+        </is>
+      </c>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E233" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="234" ht="21.95" customHeight="1">
-      <c r="C234" s="2" t="n"/>
-      <c r="D234" s="2" t="n"/>
-      <c r="E234" s="2" t="n"/>
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Sense of making an action happen</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>AGENCY</t>
+        </is>
+      </c>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E234" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="235" ht="21.95" customHeight="1">
-      <c r="C235" s="2" t="n"/>
-      <c r="D235" s="2" t="n"/>
-      <c r="E235" s="2" t="n"/>
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Shaking that may change during another
+  task</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>TREMOR</t>
+        </is>
+      </c>
+      <c r="C235" s="2" t="inlineStr"/>
+      <c r="D235" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E235" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="236" ht="21.95" customHeight="1">
-      <c r="C236" s="2" t="n"/>
-      <c r="D236" s="2" t="n"/>
-      <c r="E236" s="2" t="n"/>
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Pattern of beats examined in tremor</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>RHYTHM</t>
+        </is>
+      </c>
+      <c r="C236" s="2" t="inlineStr"/>
+      <c r="D236" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E236" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="237" ht="21.95" customHeight="1">
-      <c r="C237" s="2" t="n"/>
-      <c r="D237" s="2" t="n"/>
-      <c r="E237" s="2" t="n"/>
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Message sent between the body and brain</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>SIGNAL</t>
+        </is>
+      </c>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E237" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="238" ht="21.95" customHeight="1">
-      <c r="C238" s="2" t="n"/>
-      <c r="D238" s="2" t="n"/>
-      <c r="E238" s="2" t="n"/>
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Brain ability that may slip out of reach</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>MEMORY</t>
+        </is>
+      </c>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E238" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="239" ht="21.95" customHeight="1">
-      <c r="C239" s="2" t="n"/>
-      <c r="D239" s="2" t="n"/>
-      <c r="E239" s="2" t="n"/>
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Describes evidence gathered by the senses</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>SENSORY</t>
+        </is>
+      </c>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E239" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="240" ht="21.95" customHeight="1">
-      <c r="C240" s="2" t="n"/>
-      <c r="D240" s="2" t="n"/>
-      <c r="E240" s="2" t="n"/>
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Functional event involving altered
+  awareness or movement</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>SEIZURE</t>
+        </is>
+      </c>
+      <c r="C240" s="2" t="inlineStr"/>
+      <c r="D240" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E240" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="241" ht="21.95" customHeight="1">
-      <c r="C241" s="2" t="n"/>
-      <c r="D241" s="2" t="n"/>
-      <c r="E241" s="2" t="n"/>
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Movement can involve automatic or focused
+  forms of this</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>CONTROL</t>
+        </is>
+      </c>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E241" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="242" ht="21.95" customHeight="1">
-      <c r="C242" s="2" t="n"/>
-      <c r="D242" s="2" t="n"/>
-      <c r="E242" s="2" t="n"/>
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Messenger used alongside electrical
+  activity</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>CHEMICAL</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E242" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="243" ht="21.95" customHeight="1">
-      <c r="C243" s="2" t="n"/>
-      <c r="D243" s="2" t="n"/>
-      <c r="E243" s="2" t="n"/>
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Brain's spotlight, sometimes stolen by
+  noise</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>ATTENTION</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr"/>
+      <c r="D243" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E243" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="244" ht="21.95" customHeight="1">
-      <c r="C244" s="2" t="n"/>
-      <c r="D244" s="2" t="n"/>
-      <c r="E244" s="2" t="n"/>
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Brain's best guess about what's coming</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>PREDICTION</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E244" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="245" ht="21.95" customHeight="1">
-      <c r="C245" s="2" t="n"/>
-      <c r="D245" s="2" t="n"/>
-      <c r="E245" s="2" t="n"/>
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Movement control without step-by-step
+  planning</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>AUTOMATIC</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr"/>
+      <c r="D245" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E245" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="246" ht="21.95" customHeight="1">
-      <c r="C246" s="2" t="n"/>
-      <c r="D246" s="2" t="n"/>
-      <c r="E246" s="2" t="n"/>
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Sensing and interpreting signals inside
+  the body</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>INTEROCEPTION</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr"/>
+      <c r="D246" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E246" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="247" ht="21.95" customHeight="1">
       <c r="C247" s="2" t="n"/>

</xml_diff>

<commit_message>
Save crossword workshop question bank edits
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -5440,149 +5440,584 @@
       </c>
     </row>
     <row r="247" ht="21.95" customHeight="1">
-      <c r="C247" s="2" t="n"/>
-      <c r="D247" s="2" t="n"/>
-      <c r="E247" s="2" t="n"/>
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Even a
+  health condition that isn't FND deserves this.</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>CARE</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr"/>
+      <c r="D247" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E247" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="248" ht="21.95" customHeight="1">
-      <c r="C248" s="2" t="n"/>
-      <c r="D248" s="2" t="n"/>
-      <c r="E248" s="2" t="n"/>
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Home to
+  your muscles, bones and brain.</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>BODY</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr"/>
+      <c r="D248" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E248" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="249" ht="21.95" customHeight="1">
-      <c r="C249" s="2" t="n"/>
-      <c r="D249" s="2" t="n"/>
-      <c r="E249" s="2" t="n"/>
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Where a
+  backup ride can take you after shopping.</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>HOME</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr"/>
+      <c r="D249" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E249" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="250" ht="21.95" customHeight="1">
-      <c r="C250" s="2" t="n"/>
-      <c r="D250" s="2" t="n"/>
-      <c r="E250" s="2" t="n"/>
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>How a
+  reliable plan for getting home may help you feel.</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr"/>
+      <c r="D250" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E250" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="251" ht="21.95" customHeight="1">
-      <c r="C251" s="2" t="n"/>
-      <c r="D251" s="2" t="n"/>
-      <c r="E251" s="2" t="n"/>
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>What can
+  get easier even when symptoms stay the same.</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>LIFE</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr"/>
+      <c r="D251" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E251" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="252" ht="21.95" customHeight="1">
-      <c r="C252" s="2" t="n"/>
-      <c r="D252" s="2" t="n"/>
-      <c r="E252" s="2" t="n"/>
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Complete
+  the question: “What do we actually ___?”</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>KNOW</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr"/>
+      <c r="D252" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E252" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="253" ht="21.95" customHeight="1">
-      <c r="C253" s="2" t="n"/>
-      <c r="D253" s="2" t="n"/>
-      <c r="E253" s="2" t="n"/>
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>What
+  dimmer classroom bulbs provide less of.</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>LIGHT</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr"/>
+      <c r="D253" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E253" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="254" ht="21.95" customHeight="1">
-      <c r="C254" s="2" t="n"/>
-      <c r="D254" s="2" t="n"/>
-      <c r="E254" s="2" t="n"/>
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Where
+  grocery lists meet checkout lines.</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>STORE</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr"/>
+      <c r="D254" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E254" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="255" ht="21.95" customHeight="1">
-      <c r="C255" s="2" t="n"/>
-      <c r="D255" s="2" t="n"/>
-      <c r="E255" s="2" t="n"/>
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>An
+  informal word for a sudden worsening after exceeding your limit.</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr"/>
+      <c r="D255" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E255" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="256" ht="21.95" customHeight="1">
-      <c r="C256" s="2" t="n"/>
-      <c r="D256" s="2" t="n"/>
-      <c r="E256" s="2" t="n"/>
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Good
+  support should fit a person's individual ___.</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>NEEDS</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr"/>
+      <c r="D256" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E256" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="257" ht="21.95" customHeight="1">
-      <c r="C257" s="2" t="n"/>
-      <c r="D257" s="2" t="n"/>
-      <c r="E257" s="2" t="n"/>
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Things
+  we can confirm, rather than just guess.</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>FACTS</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr"/>
+      <c r="D257" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E257" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="258" ht="21.95" customHeight="1">
-      <c r="C258" s="2" t="n"/>
-      <c r="D258" s="2" t="n"/>
-      <c r="E258" s="2" t="n"/>
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Sleep,
+  pain and illness can all affect this.</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>HEALTH</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr"/>
+      <c r="D258" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E258" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="259" ht="21.95" customHeight="1">
-      <c r="C259" s="2" t="n"/>
-      <c r="D259" s="2" t="n"/>
-      <c r="E259" s="2" t="n"/>
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>A place
+  to get treatment, not groceries.</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>CLINIC</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr"/>
+      <c r="D259" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E259" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="260" ht="21.95" customHeight="1">
-      <c r="C260" s="2" t="n"/>
-      <c r="D260" s="2" t="n"/>
-      <c r="E260" s="2" t="n"/>
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>A backup
+  ride gives you another one of these.</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>OPTION</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr"/>
+      <c r="D260" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E260" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="261" ht="21.95" customHeight="1">
-      <c r="C261" s="2" t="n"/>
-      <c r="D261" s="2" t="n"/>
-      <c r="E261" s="2" t="n"/>
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>A
+  shopping trip or other journey away from home.</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>OUTING</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr"/>
+      <c r="D261" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E261" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="262" ht="21.95" customHeight="1">
-      <c r="C262" s="2" t="n"/>
-      <c r="D262" s="2" t="n"/>
-      <c r="E262" s="2" t="n"/>
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Physical
+  harm sometimes investigated as a possible FND trigger.</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>INJURY</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr"/>
+      <c r="D262" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E262" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="263" ht="21.95" customHeight="1">
-      <c r="C263" s="2" t="n"/>
-      <c r="D263" s="2" t="n"/>
-      <c r="E263" s="2" t="n"/>
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Make a
+  task more manageable</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>ADJUST</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr"/>
+      <c r="D263" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E263" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="264" ht="21.95" customHeight="1">
-      <c r="C264" s="2" t="n"/>
-      <c r="D264" s="2" t="n"/>
-      <c r="E264" s="2" t="n"/>
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>A small
+  slice of time that can strengthen a relationship.</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>MOMENT</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr"/>
+      <c r="D264" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E264" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="265" ht="21.95" customHeight="1">
-      <c r="C265" s="2" t="n"/>
-      <c r="D265" s="2" t="n"/>
-      <c r="E265" s="2" t="n"/>
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Research
+  results, rather than educated guesses.</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>FINDINGS</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr"/>
+      <c r="D265" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E265" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="266" ht="21.95" customHeight="1">
-      <c r="C266" s="2" t="n"/>
-      <c r="D266" s="2" t="n"/>
-      <c r="E266" s="2" t="n"/>
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Something
+  experienced with a health condition, such as pain or weakness.</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>SYMPTOM</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr"/>
+      <c r="D266" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E266" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="267" ht="21.95" customHeight="1">
-      <c r="C267" s="2" t="n"/>
-      <c r="D267" s="2" t="n"/>
-      <c r="E267" s="2" t="n"/>
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>A health
+  worry worth discussing with your clinician.</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>CONCERN</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr"/>
+      <c r="D267" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E267" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="268" ht="21.95" customHeight="1">
-      <c r="C268" s="2" t="n"/>
-      <c r="D268" s="2" t="n"/>
-      <c r="E268" s="2" t="n"/>
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>What
+  daily life can do even when symptoms remain.</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>IMPROVE</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr"/>
+      <c r="D268" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E268" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="269" ht="21.95" customHeight="1">
-      <c r="C269" s="2" t="n"/>
-      <c r="D269" s="2" t="n"/>
-      <c r="E269" s="2" t="n"/>
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Physical,
+  psychological and social influences on daily life.</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>FACTORS</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr"/>
+      <c r="D269" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E269" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="270" ht="21.95" customHeight="1">
-      <c r="C270" s="2" t="n"/>
-      <c r="D270" s="2" t="n"/>
-      <c r="E270" s="2" t="n"/>
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>A
+  clinician's identification of a condition, not a whole life story.</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>DIAGNOSIS</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr"/>
+      <c r="D270" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E270" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="271" ht="21.95" customHeight="1">
-      <c r="C271" s="2" t="n"/>
-      <c r="D271" s="2" t="n"/>
-      <c r="E271" s="2" t="n"/>
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>A
+  personal limit beyond which someone may experience a crash.</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr"/>
+      <c r="D271" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E271" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="272" ht="21.95" customHeight="1">
-      <c r="C272" s="2" t="n"/>
-      <c r="D272" s="2" t="n"/>
-      <c r="E272" s="2" t="n"/>
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Hobbies,
+  errands and outings are examples of these.</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>ACTIVITIES</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr"/>
+      <c r="D272" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E272" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="273" ht="21.95" customHeight="1">
-      <c r="C273" s="2" t="n"/>
-      <c r="D273" s="2" t="n"/>
-      <c r="E273" s="2" t="n"/>
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>People
+  investigating possible FND connections instead of guessing.</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>SCIENTISTS</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr"/>
+      <c r="D273" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E273" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="274" ht="21.95" customHeight="1">
-      <c r="C274" s="2" t="n"/>
-      <c r="D274" s="2" t="n"/>
-      <c r="E274" s="2" t="n"/>
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>A
+  suggested account of why something happened.</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>EXPLANATION</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr"/>
+      <c r="D274" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E274" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="275" ht="21.95" customHeight="1">
-      <c r="C275" s="2" t="n"/>
-      <c r="D275" s="2" t="n"/>
-      <c r="E275" s="2" t="n"/>
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Lights,
+  noises and places around you are all part of these.</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>SURROUNDINGS</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr"/>
+      <c r="D275" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E275" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="276" ht="21.95" customHeight="1">
       <c r="C276" s="2" t="n"/>

</xml_diff>

<commit_message>
Crossword workshop question bank — 2026-10-21 (#170)
Saved Excel question-bank edits from the Codespaces crossword workshop.
Review and merge manually. Finished puzzle PDFs are published
separately.
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -5440,149 +5440,584 @@
       </c>
     </row>
     <row r="247" ht="21.95" customHeight="1">
-      <c r="C247" s="2" t="n"/>
-      <c r="D247" s="2" t="n"/>
-      <c r="E247" s="2" t="n"/>
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Even a
+  health condition that isn't FND deserves this.</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>CARE</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr"/>
+      <c r="D247" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E247" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="248" ht="21.95" customHeight="1">
-      <c r="C248" s="2" t="n"/>
-      <c r="D248" s="2" t="n"/>
-      <c r="E248" s="2" t="n"/>
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Home to
+  your muscles, bones and brain.</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>BODY</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr"/>
+      <c r="D248" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E248" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="249" ht="21.95" customHeight="1">
-      <c r="C249" s="2" t="n"/>
-      <c r="D249" s="2" t="n"/>
-      <c r="E249" s="2" t="n"/>
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Where a
+  backup ride can take you after shopping.</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>HOME</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr"/>
+      <c r="D249" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E249" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="250" ht="21.95" customHeight="1">
-      <c r="C250" s="2" t="n"/>
-      <c r="D250" s="2" t="n"/>
-      <c r="E250" s="2" t="n"/>
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>How a
+  reliable plan for getting home may help you feel.</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr"/>
+      <c r="D250" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E250" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="251" ht="21.95" customHeight="1">
-      <c r="C251" s="2" t="n"/>
-      <c r="D251" s="2" t="n"/>
-      <c r="E251" s="2" t="n"/>
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>What can
+  get easier even when symptoms stay the same.</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>LIFE</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr"/>
+      <c r="D251" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E251" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="252" ht="21.95" customHeight="1">
-      <c r="C252" s="2" t="n"/>
-      <c r="D252" s="2" t="n"/>
-      <c r="E252" s="2" t="n"/>
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Complete
+  the question: “What do we actually ___?”</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>KNOW</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr"/>
+      <c r="D252" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E252" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="253" ht="21.95" customHeight="1">
-      <c r="C253" s="2" t="n"/>
-      <c r="D253" s="2" t="n"/>
-      <c r="E253" s="2" t="n"/>
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>What
+  dimmer classroom bulbs provide less of.</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>LIGHT</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr"/>
+      <c r="D253" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E253" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="254" ht="21.95" customHeight="1">
-      <c r="C254" s="2" t="n"/>
-      <c r="D254" s="2" t="n"/>
-      <c r="E254" s="2" t="n"/>
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Where
+  grocery lists meet checkout lines.</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>STORE</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr"/>
+      <c r="D254" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E254" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="255" ht="21.95" customHeight="1">
-      <c r="C255" s="2" t="n"/>
-      <c r="D255" s="2" t="n"/>
-      <c r="E255" s="2" t="n"/>
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>An
+  informal word for a sudden worsening after exceeding your limit.</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>CRASH</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr"/>
+      <c r="D255" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E255" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="256" ht="21.95" customHeight="1">
-      <c r="C256" s="2" t="n"/>
-      <c r="D256" s="2" t="n"/>
-      <c r="E256" s="2" t="n"/>
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Good
+  support should fit a person's individual ___.</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>NEEDS</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr"/>
+      <c r="D256" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E256" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="257" ht="21.95" customHeight="1">
-      <c r="C257" s="2" t="n"/>
-      <c r="D257" s="2" t="n"/>
-      <c r="E257" s="2" t="n"/>
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Things
+  we can confirm, rather than just guess.</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>FACTS</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr"/>
+      <c r="D257" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E257" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="258" ht="21.95" customHeight="1">
-      <c r="C258" s="2" t="n"/>
-      <c r="D258" s="2" t="n"/>
-      <c r="E258" s="2" t="n"/>
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Sleep,
+  pain and illness can all affect this.</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>HEALTH</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr"/>
+      <c r="D258" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E258" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="259" ht="21.95" customHeight="1">
-      <c r="C259" s="2" t="n"/>
-      <c r="D259" s="2" t="n"/>
-      <c r="E259" s="2" t="n"/>
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>A place
+  to get treatment, not groceries.</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>CLINIC</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr"/>
+      <c r="D259" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E259" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="260" ht="21.95" customHeight="1">
-      <c r="C260" s="2" t="n"/>
-      <c r="D260" s="2" t="n"/>
-      <c r="E260" s="2" t="n"/>
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>A backup
+  ride gives you another one of these.</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>OPTION</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr"/>
+      <c r="D260" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E260" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="261" ht="21.95" customHeight="1">
-      <c r="C261" s="2" t="n"/>
-      <c r="D261" s="2" t="n"/>
-      <c r="E261" s="2" t="n"/>
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>A
+  shopping trip or other journey away from home.</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>OUTING</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr"/>
+      <c r="D261" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E261" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="262" ht="21.95" customHeight="1">
-      <c r="C262" s="2" t="n"/>
-      <c r="D262" s="2" t="n"/>
-      <c r="E262" s="2" t="n"/>
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Physical
+  harm sometimes investigated as a possible FND trigger.</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>INJURY</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr"/>
+      <c r="D262" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E262" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="263" ht="21.95" customHeight="1">
-      <c r="C263" s="2" t="n"/>
-      <c r="D263" s="2" t="n"/>
-      <c r="E263" s="2" t="n"/>
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Make a
+  task more manageable</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>ADJUST</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr"/>
+      <c r="D263" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E263" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="264" ht="21.95" customHeight="1">
-      <c r="C264" s="2" t="n"/>
-      <c r="D264" s="2" t="n"/>
-      <c r="E264" s="2" t="n"/>
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>A small
+  slice of time that can strengthen a relationship.</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>MOMENT</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr"/>
+      <c r="D264" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E264" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="265" ht="21.95" customHeight="1">
-      <c r="C265" s="2" t="n"/>
-      <c r="D265" s="2" t="n"/>
-      <c r="E265" s="2" t="n"/>
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Research
+  results, rather than educated guesses.</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>FINDINGS</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr"/>
+      <c r="D265" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E265" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="266" ht="21.95" customHeight="1">
-      <c r="C266" s="2" t="n"/>
-      <c r="D266" s="2" t="n"/>
-      <c r="E266" s="2" t="n"/>
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Something
+  experienced with a health condition, such as pain or weakness.</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>SYMPTOM</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr"/>
+      <c r="D266" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E266" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="267" ht="21.95" customHeight="1">
-      <c r="C267" s="2" t="n"/>
-      <c r="D267" s="2" t="n"/>
-      <c r="E267" s="2" t="n"/>
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>A health
+  worry worth discussing with your clinician.</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>CONCERN</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr"/>
+      <c r="D267" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E267" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="268" ht="21.95" customHeight="1">
-      <c r="C268" s="2" t="n"/>
-      <c r="D268" s="2" t="n"/>
-      <c r="E268" s="2" t="n"/>
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>What
+  daily life can do even when symptoms remain.</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>IMPROVE</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr"/>
+      <c r="D268" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E268" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="269" ht="21.95" customHeight="1">
-      <c r="C269" s="2" t="n"/>
-      <c r="D269" s="2" t="n"/>
-      <c r="E269" s="2" t="n"/>
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Physical,
+  psychological and social influences on daily life.</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>FACTORS</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr"/>
+      <c r="D269" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E269" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="270" ht="21.95" customHeight="1">
-      <c r="C270" s="2" t="n"/>
-      <c r="D270" s="2" t="n"/>
-      <c r="E270" s="2" t="n"/>
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>A
+  clinician's identification of a condition, not a whole life story.</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>DIAGNOSIS</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr"/>
+      <c r="D270" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E270" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="271" ht="21.95" customHeight="1">
-      <c r="C271" s="2" t="n"/>
-      <c r="D271" s="2" t="n"/>
-      <c r="E271" s="2" t="n"/>
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>A
+  personal limit beyond which someone may experience a crash.</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>THRESHOLD</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr"/>
+      <c r="D271" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E271" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="272" ht="21.95" customHeight="1">
-      <c r="C272" s="2" t="n"/>
-      <c r="D272" s="2" t="n"/>
-      <c r="E272" s="2" t="n"/>
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Hobbies,
+  errands and outings are examples of these.</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>ACTIVITIES</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr"/>
+      <c r="D272" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E272" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="273" ht="21.95" customHeight="1">
-      <c r="C273" s="2" t="n"/>
-      <c r="D273" s="2" t="n"/>
-      <c r="E273" s="2" t="n"/>
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>People
+  investigating possible FND connections instead of guessing.</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>SCIENTISTS</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr"/>
+      <c r="D273" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E273" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="274" ht="21.95" customHeight="1">
-      <c r="C274" s="2" t="n"/>
-      <c r="D274" s="2" t="n"/>
-      <c r="E274" s="2" t="n"/>
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>A
+  suggested account of why something happened.</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>EXPLANATION</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr"/>
+      <c r="D274" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E274" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="275" ht="21.95" customHeight="1">
-      <c r="C275" s="2" t="n"/>
-      <c r="D275" s="2" t="n"/>
-      <c r="E275" s="2" t="n"/>
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Lights,
+  noises and places around you are all part of these.</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>SURROUNDINGS</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr"/>
+      <c r="D275" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E275" s="2" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="276" ht="21.95" customHeight="1">
       <c r="C276" s="2" t="n"/>

</xml_diff>

<commit_message>
Crossword workshop question bank — 2026-10-23 (#179)
Saved Excel question-bank edits from the Codespaces crossword workshop.
Review and merge manually. Finished puzzle PDFs are published
separately.
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -6020,179 +6020,764 @@
       </c>
     </row>
     <row r="276" ht="21.95" customHeight="1">
-      <c r="C276" s="2" t="n"/>
-      <c r="D276" s="2" t="n"/>
-      <c r="E276" s="2" t="n"/>
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>A small
+  guide to your health, rather than a hunt for buried treasure.</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>MAP</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E276" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="277" ht="21.95" customHeight="1">
-      <c r="C277" s="2" t="n"/>
-      <c r="D277" s="2" t="n"/>
-      <c r="E277" s="2" t="n"/>
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Three-letter
+  abbreviation for functional neurological disorder.</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>FND</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr"/>
+      <c r="D277" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E277" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="278" ht="21.95" customHeight="1">
-      <c r="C278" s="2" t="n"/>
-      <c r="D278" s="2" t="n"/>
-      <c r="E278" s="2" t="n"/>
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Body
+  part that may experience functional weakness, below the hip.</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>LEG</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr"/>
+      <c r="D278" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E278" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="279" ht="21.95" customHeight="1">
-      <c r="C279" s="2" t="n"/>
-      <c r="D279" s="2" t="n"/>
-      <c r="E279" s="2" t="n"/>
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>A few
+  written words that save your memory some work.</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>NOTE</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr"/>
+      <c r="D279" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E279" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="280" ht="21.95" customHeight="1">
-      <c r="C280" s="2" t="n"/>
-      <c r="D280" s="2" t="n"/>
-      <c r="E280" s="2" t="n"/>
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>What a
+  new, serious health problem may need promptly.</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>CARE</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr"/>
+      <c r="D280" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E280" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="281" ht="21.95" customHeight="1">
-      <c r="C281" s="2" t="n"/>
-      <c r="D281" s="2" t="n"/>
-      <c r="E281" s="2" t="n"/>
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Assistance
+  when managing something alone gets difficult.</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>HELP</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr"/>
+      <c r="D281" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E281" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="282" ht="21.95" customHeight="1">
-      <c r="C282" s="2" t="n"/>
-      <c r="D282" s="2" t="n"/>
-      <c r="E282" s="2" t="n"/>
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>What
+  gets muddled when two weeks ago feels like four months ago.</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E282" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="283" ht="21.95" customHeight="1">
-      <c r="C283" s="2" t="n"/>
-      <c r="D283" s="2" t="n"/>
-      <c r="E283" s="2" t="n"/>
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>An
+  increased chance of something happening, rather than a certainty.</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>RISK</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E283" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="284" ht="21.95" customHeight="1">
-      <c r="C284" s="2" t="n"/>
-      <c r="D284" s="2" t="n"/>
-      <c r="E284" s="2" t="n"/>
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>A poor
+  night of this might come before a difficult day.</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>SLEEP</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr"/>
+      <c r="D284" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E284" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="285" ht="21.95" customHeight="1">
-      <c r="C285" s="2" t="n"/>
-      <c r="D285" s="2" t="n"/>
-      <c r="E285" s="2" t="n"/>
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Describes
+  something already established, rather than still uncertain.</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>KNOWN</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr"/>
+      <c r="D285" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E285" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="286" ht="21.95" customHeight="1">
-      <c r="C286" s="2" t="n"/>
-      <c r="D286" s="2" t="n"/>
-      <c r="E286" s="2" t="n"/>
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Your
+  thinking headquarters, occasionally a little forgetful.</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>BRAIN</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E286" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="287" ht="21.95" customHeight="1">
-      <c r="C287" s="2" t="n"/>
-      <c r="D287" s="2" t="n"/>
-      <c r="E287" s="2" t="n"/>
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Sometimes
+  the hardest things to find during a doctor's appointment.</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>WORDS</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E287" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="288" ht="21.95" customHeight="1">
-      <c r="C288" s="2" t="n"/>
-      <c r="D288" s="2" t="n"/>
-      <c r="E288" s="2" t="n"/>
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Talking
+  ability that may change around a functional episode.</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>SPEECH</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr"/>
+      <c r="D288" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E288" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="289" ht="21.95" customHeight="1">
-      <c r="C289" s="2" t="n"/>
-      <c r="D289" s="2" t="n"/>
-      <c r="E289" s="2" t="n"/>
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>The
+  mental filing cabinet that sometimes misplaces dates.</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>MEMORY</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E289" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="290" ht="21.95" customHeight="1">
-      <c r="C290" s="2" t="n"/>
-      <c r="D290" s="2" t="n"/>
-      <c r="E290" s="2" t="n"/>
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>The
+  bigger picture that includes FND and other conditions.</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>HEALTH</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr"/>
+      <c r="D290" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E290" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="291" ht="21.95" customHeight="1">
-      <c r="C291" s="2" t="n"/>
-      <c r="D291" s="2" t="n"/>
-      <c r="E291" s="2" t="n"/>
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>A
+  written account that helps when details escape you.</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>RECORD</t>
+        </is>
+      </c>
+      <c r="C291" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E291" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="292" ht="21.95" customHeight="1">
-      <c r="C292" s="2" t="n"/>
-      <c r="D292" s="2" t="n"/>
-      <c r="E292" s="2" t="n"/>
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>A
+  possible influence, as in a risk or maintaining ___.</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>FACTOR</t>
+        </is>
+      </c>
+      <c r="C292" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E292" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="293" ht="21.95" customHeight="1">
-      <c r="C293" s="2" t="n"/>
-      <c r="D293" s="2" t="n"/>
-      <c r="E293" s="2" t="n"/>
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>A
+  difference from your usual symptoms that may be worth mentioning.</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>CHANGE</t>
+        </is>
+      </c>
+      <c r="C293" s="2" t="inlineStr"/>
+      <c r="D293" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E293" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="294" ht="21.95" customHeight="1">
-      <c r="C294" s="2" t="n"/>
-      <c r="D294" s="2" t="n"/>
-      <c r="E294" s="2" t="n"/>
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>A
+  medical professional you may visit for an appointment.</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>DOCTOR</t>
+        </is>
+      </c>
+      <c r="C294" s="2" t="inlineStr"/>
+      <c r="D294" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E294" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="295" ht="21.95" customHeight="1">
-      <c r="C295" s="2" t="n"/>
-      <c r="D295" s="2" t="n"/>
-      <c r="E295" s="2" t="n"/>
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>When a
+  possible trigger happens relative to an episode.</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>BEFORE</t>
+        </is>
+      </c>
+      <c r="C295" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E295" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="296" ht="21.95" customHeight="1">
-      <c r="C296" s="2" t="n"/>
-      <c r="D296" s="2" t="n"/>
-      <c r="E296" s="2" t="n"/>
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>The
+  middle part of a sequence: before, ___, after.</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>DURING</t>
+        </is>
+      </c>
+      <c r="C296" s="2" t="inlineStr"/>
+      <c r="D296" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E296" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="297" ht="21.95" customHeight="1">
-      <c r="C297" s="2" t="n"/>
-      <c r="D297" s="2" t="n"/>
-      <c r="E297" s="2" t="n"/>
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>A
+  possible spark that increases the chance of symptoms.</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>TRIGGER</t>
+        </is>
+      </c>
+      <c r="C297" s="2" t="inlineStr"/>
+      <c r="D297" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E297" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="298" ht="21.95" customHeight="1">
-      <c r="C298" s="2" t="n"/>
-      <c r="D298" s="2" t="n"/>
-      <c r="E298" s="2" t="n"/>
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Type of
+  sign that may suggest a familiar episode is beginning.</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C298" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E298" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="299" ht="21.95" customHeight="1">
-      <c r="C299" s="2" t="n"/>
-      <c r="D299" s="2" t="n"/>
-      <c r="E299" s="2" t="n"/>
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>A period
+  when symptoms occur, rather than remaining continuously present.</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>EPISODE</t>
+        </is>
+      </c>
+      <c r="C299" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E299" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="300" ht="21.95" customHeight="1">
-      <c r="C300" s="2" t="n"/>
-      <c r="D300" s="2" t="n"/>
-      <c r="E300" s="2" t="n"/>
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Something
+  repeated that gives clues, but doesn't automatically prove a cause.</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>PATTERN</t>
+        </is>
+      </c>
+      <c r="C300" s="2" t="inlineStr"/>
+      <c r="D300" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E300" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="301" ht="21.95" customHeight="1">
-      <c r="C301" s="2" t="n"/>
-      <c r="D301" s="2" t="n"/>
-      <c r="E301" s="2" t="n"/>
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>An
+  experienced health difficulty, such as weakness or dizziness.</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>SYMPTOM</t>
+        </is>
+      </c>
+      <c r="C301" s="2" t="inlineStr"/>
+      <c r="D301" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E301" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="302" ht="21.95" customHeight="1">
-      <c r="C302" s="2" t="n"/>
-      <c r="D302" s="2" t="n"/>
-      <c r="E302" s="2" t="n"/>
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>A
+  neurological condition that can coexist with FND and cause head pain.</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>MIGRAINE</t>
+        </is>
+      </c>
+      <c r="C302" s="2" t="inlineStr"/>
+      <c r="D302" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E302" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="303" ht="21.95" customHeight="1">
-      <c r="C303" s="2" t="n"/>
-      <c r="D303" s="2" t="n"/>
-      <c r="E303" s="2" t="n"/>
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Reduced
+  strength that may sometimes be diagnosed as functional.</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>WEAKNESS</t>
+        </is>
+      </c>
+      <c r="C303" s="2" t="inlineStr"/>
+      <c r="D303" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E303" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="304" ht="21.95" customHeight="1">
-      <c r="C304" s="2" t="n"/>
-      <c r="D304" s="2" t="n"/>
-      <c r="E304" s="2" t="n"/>
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Feeling
+  lightheaded or unsteady, sometimes a new medical question.</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>DIZZINESS</t>
+        </is>
+      </c>
+      <c r="C304" s="2" t="inlineStr"/>
+      <c r="D304" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E304" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="305" ht="21.95" customHeight="1">
-      <c r="C305" s="2" t="n"/>
-      <c r="D305" s="2" t="n"/>
-      <c r="E305" s="2" t="n"/>
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>The
+  identification of a medical condition following clinical assessment.</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>DIAGNOSIS</t>
+        </is>
+      </c>
+      <c r="C305" s="2" t="inlineStr"/>
+      <c r="D305" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E305" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="306" ht="21.95" customHeight="1">
-      <c r="C306" s="2" t="n"/>
-      <c r="D306" s="2" t="n"/>
-      <c r="E306" s="2" t="n"/>
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Healthcare
+  professional who assesses symptoms and may make diagnoses.</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>CLINICIAN</t>
+        </is>
+      </c>
+      <c r="C306" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E306" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="307" ht="21.95" customHeight="1">
-      <c r="C307" s="2" t="n"/>
-      <c r="D307" s="2" t="n"/>
-      <c r="E307" s="2" t="n"/>
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>A
+  clinical evaluation to investigate or understand a symptom.</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>ASSESSMENT</t>
+        </is>
+      </c>
+      <c r="C307" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E307" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="308" ht="21.95" customHeight="1">
-      <c r="C308" s="2" t="n"/>
-      <c r="D308" s="2" t="n"/>
-      <c r="E308" s="2" t="n"/>
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Medical
+  term for a condition occurring alongside another condition.</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>COMORBIDITY</t>
+        </is>
+      </c>
+      <c r="C308" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E308" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="309" ht="21.95" customHeight="1">
-      <c r="C309" s="2" t="n"/>
-      <c r="D309" s="2" t="n"/>
-      <c r="E309" s="2" t="n"/>
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Something
+  that follows an episode, possibly including exhaustion.</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>CONSEQUENCE</t>
+        </is>
+      </c>
+      <c r="C309" s="2" t="inlineStr"/>
+      <c r="D309" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E309" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="310" ht="21.95" customHeight="1">
-      <c r="C310" s="2" t="n"/>
-      <c r="D310" s="2" t="n"/>
-      <c r="E310" s="2" t="n"/>
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Type of
+  factor that may contribute to symptoms continuing.</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>MAINTAINING</t>
+        </is>
+      </c>
+      <c r="C310" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E310" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="311" ht="21.95" customHeight="1">
       <c r="C311" s="2" t="n"/>

</xml_diff>

<commit_message>
Crossword workshop question bank — 2026-10-23 (#182)
Saved Excel question-bank edits from the Codespaces crossword workshop.
Review and merge manually. Finished puzzle PDFs are published
separately.
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -6780,154 +6780,651 @@
       </c>
     </row>
     <row r="311" ht="21.95" customHeight="1">
-      <c r="C311" s="2" t="n"/>
-      <c r="D311" s="2" t="n"/>
-      <c r="E311" s="2" t="n"/>
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>A
+  helpful tool that makes an activity easier.</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>AID</t>
+        </is>
+      </c>
+      <c r="C311" s="2" t="inlineStr"/>
+      <c r="D311" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E311" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="312" ht="21.95" customHeight="1">
-      <c r="C312" s="2" t="n"/>
-      <c r="D312" s="2" t="n"/>
-      <c r="E312" s="2" t="n"/>
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Belonging
+  to you, rather than borrowed.</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>OWN</t>
+        </is>
+      </c>
+      <c r="C312" s="2" t="inlineStr"/>
+      <c r="D312" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E312" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="313" ht="21.95" customHeight="1">
-      <c r="C313" s="2" t="n"/>
-      <c r="D313" s="2" t="n"/>
-      <c r="E313" s="2" t="n"/>
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>A
+  24-hour slice of life.</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>DAY</t>
+        </is>
+      </c>
+      <c r="C313" s="2" t="inlineStr"/>
+      <c r="D313" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E313" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="314" ht="21.95" customHeight="1">
-      <c r="C314" s="2" t="n"/>
-      <c r="D314" s="2" t="n"/>
-      <c r="E314" s="2" t="n"/>
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>One ____
+  may hold an entire health summary.</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>PAGE</t>
+        </is>
+      </c>
+      <c r="C314" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E314" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="315" ht="21.95" customHeight="1">
-      <c r="C315" s="2" t="n"/>
-      <c r="D315" s="2" t="n"/>
-      <c r="E315" s="2" t="n"/>
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>A chance
+  to recharge between demanding activities.</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="C315" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E315" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="316" ht="21.95" customHeight="1">
-      <c r="C316" s="2" t="n"/>
-      <c r="D316" s="2" t="n"/>
-      <c r="E316" s="2" t="n"/>
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>A piece
+  of work to finish.</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>TASK</t>
+        </is>
+      </c>
+      <c r="C316" s="2" t="inlineStr"/>
+      <c r="D316" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E316" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="317" ht="21.95" customHeight="1">
-      <c r="C317" s="2" t="n"/>
-      <c r="D317" s="2" t="n"/>
-      <c r="E317" s="2" t="n"/>
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>A hint
+  worth exploring, rather than proof.</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>CLUE</t>
+        </is>
+      </c>
+      <c r="C317" s="2" t="inlineStr"/>
+      <c r="D317" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E317" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="318" ht="21.95" customHeight="1">
-      <c r="C318" s="2" t="n"/>
-      <c r="D318" s="2" t="n"/>
-      <c r="E318" s="2" t="n"/>
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>A dated
+  record of daily experiences.</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>DIARY</t>
+        </is>
+      </c>
+      <c r="C318" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E318" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="319" ht="21.95" customHeight="1">
-      <c r="C319" s="2" t="n"/>
-      <c r="D319" s="2" t="n"/>
-      <c r="E319" s="2" t="n"/>
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Peaceful.</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>QUIET</t>
+        </is>
+      </c>
+      <c r="C319" s="2" t="inlineStr"/>
+      <c r="D319" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E319" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="320" ht="21.95" customHeight="1">
-      <c r="C320" s="2" t="n"/>
-      <c r="D320" s="2" t="n"/>
-      <c r="E320" s="2" t="n"/>
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Old-school
+  writing surface. No batteries required!</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr"/>
+      <c r="D320" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E320" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="321" ht="21.95" customHeight="1">
-      <c r="C321" s="2" t="n"/>
-      <c r="D321" s="2" t="n"/>
-      <c r="E321" s="2" t="n"/>
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>A
+  planned pause</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>BREAK</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E321" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="322" ht="21.95" customHeight="1">
-      <c r="C322" s="2" t="n"/>
-      <c r="D322" s="2" t="n"/>
-      <c r="E322" s="2" t="n"/>
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>The aim
+  of planning for risks and getting help.</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>SAFETY</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr"/>
+      <c r="D322" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E322" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="323" ht="21.95" customHeight="1">
-      <c r="C323" s="2" t="n"/>
-      <c r="D323" s="2" t="n"/>
-      <c r="E323" s="2" t="n"/>
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Perhaps
+  made easier by an aid.</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>OUTING</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E323" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="324" ht="21.95" customHeight="1">
-      <c r="C324" s="2" t="n"/>
-      <c r="D324" s="2" t="n"/>
-      <c r="E324" s="2" t="n"/>
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Look
+  over information again to see what matters.</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr"/>
+      <c r="D324" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E324" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="325" ht="21.95" customHeight="1">
-      <c r="C325" s="2" t="n"/>
-      <c r="D325" s="2" t="n"/>
-      <c r="E325" s="2" t="n"/>
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Practical
+  assistance that makes life more manageable.</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>SUPPORT</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr"/>
+      <c r="D325" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E325" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="326" ht="21.95" customHeight="1">
-      <c r="C326" s="2" t="n"/>
-      <c r="D326" s="2" t="n"/>
-      <c r="E326" s="2" t="n"/>
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Something
+  you can do, even when it comes and goes.</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>ABILITY</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E326" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="327" ht="21.95" customHeight="1">
-      <c r="C327" s="2" t="n"/>
-      <c r="D327" s="2" t="n"/>
-      <c r="E327" s="2" t="n"/>
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Relating
+  to touch, sound, sight or other senses.</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>SENSORY</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr"/>
+      <c r="D327" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E327" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="328" ht="21.95" customHeight="1">
-      <c r="C328" s="2" t="n"/>
-      <c r="D328" s="2" t="n"/>
-      <c r="E328" s="2" t="n"/>
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Briefly
+  recording changes to answer a question.</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>TRACKING</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E328" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="329" ht="21.95" customHeight="1">
-      <c r="C329" s="2" t="n"/>
-      <c r="D329" s="2" t="n"/>
-      <c r="E329" s="2" t="n"/>
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>A
+  helpful nudge for a forgetful moment.</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>REMINDER</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E329" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="330" ht="21.95" customHeight="1">
-      <c r="C330" s="2" t="n"/>
-      <c r="D330" s="2" t="n"/>
-      <c r="E330" s="2" t="n"/>
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>The
+  process of regaining strength after a demanding event.</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>RECOVERY</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr"/>
+      <c r="D330" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E330" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="331" ht="21.95" customHeight="1">
-      <c r="C331" s="2" t="n"/>
-      <c r="D331" s="2" t="n"/>
-      <c r="E331" s="2" t="n"/>
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Changes
+  in this may be part of someone's FND.</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>MOVEMENT</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr"/>
+      <c r="D331" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E331" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="332" ht="21.95" customHeight="1">
-      <c r="C332" s="2" t="n"/>
-      <c r="D332" s="2" t="n"/>
-      <c r="E332" s="2" t="n"/>
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>A
+  practical approach to making something easier.</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>STRATEGY</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E332" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="333" ht="21.95" customHeight="1">
-      <c r="C333" s="2" t="n"/>
-      <c r="D333" s="2" t="n"/>
-      <c r="E333" s="2" t="n"/>
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Able to
+  happen or be done, perhaps with an adjustment.</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>POSSIBLE</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E333" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="334" ht="21.95" customHeight="1">
-      <c r="C334" s="2" t="n"/>
-      <c r="D334" s="2" t="n"/>
-      <c r="E334" s="2" t="n"/>
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Some
+  people with FND experience functional ___.</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>SEIZURES</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr"/>
+      <c r="D334" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E334" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="335" ht="21.95" customHeight="1">
-      <c r="C335" s="2" t="n"/>
-      <c r="D335" s="2" t="n"/>
-      <c r="E335" s="2" t="n"/>
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>People
+  connected through shared interests or experiences.</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>COMMUNITY</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr"/>
+      <c r="D335" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E335" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="336" ht="21.95" customHeight="1">
-      <c r="C336" s="2" t="n"/>
-      <c r="D336" s="2" t="n"/>
-      <c r="E336" s="2" t="n"/>
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Relating
+  to thinking, memory and attention.</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>COGNITIVE</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E336" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="337" ht="21.95" customHeight="1">
-      <c r="C337" s="2" t="n"/>
-      <c r="D337" s="2" t="n"/>
-      <c r="E337" s="2" t="n"/>
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>An
+  empty-battery kind of feeling.</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>EXHAUSTED</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr"/>
+      <c r="D337" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E337" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="338" ht="21.95" customHeight="1">
-      <c r="C338" s="2" t="n"/>
-      <c r="D338" s="2" t="n"/>
-      <c r="E338" s="2" t="n"/>
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>A
+  helpful change to a setting or routine.</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>ADJUSTMENT</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E338" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="339" ht="21.95" customHeight="1">
-      <c r="C339" s="2" t="n"/>
-      <c r="D339" s="2" t="n"/>
-      <c r="E339" s="2" t="n"/>
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Facts
+  and details that help explain a situation.</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>INFORMATION</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr"/>
+      <c r="D339" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E339" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="340" ht="21.95" customHeight="1">
-      <c r="C340" s="2" t="n"/>
-      <c r="D340" s="2" t="n"/>
-      <c r="E340" s="2" t="n"/>
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Everything
+  around you, including light and noise.</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>SURROUNDINGS</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr"/>
+      <c r="D340" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E340" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="341" ht="21.95" customHeight="1">
       <c r="C341" s="2" t="n"/>

</xml_diff>

<commit_message>
Crossword workshop question bank — 2026-10-25 (#188)
Saved Excel question-bank edits from the Codespaces crossword workshop.
Review and merge manually. Finished puzzle PDFs are published
separately.
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -370,7 +370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E401"/>
+  <dimension ref="A1:E445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="70.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -7427,309 +7427,2312 @@
       </c>
     </row>
     <row r="341" ht="21.95" customHeight="1">
-      <c r="C341" s="2" t="n"/>
-      <c r="D341" s="2" t="n"/>
-      <c r="E341" s="2" t="n"/>
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>A
+  symptom never experienced before</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D341" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E341" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="342" ht="21.95" customHeight="1">
-      <c r="C342" s="2" t="n"/>
-      <c r="D342" s="2" t="n"/>
-      <c r="E342" s="2" t="n"/>
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>What a
+  trembling hand does</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>SHAKE</t>
+        </is>
+      </c>
+      <c r="C342" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D342" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E342" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="343" ht="21.95" customHeight="1">
-      <c r="C343" s="2" t="n"/>
-      <c r="D343" s="2" t="n"/>
-      <c r="E343" s="2" t="n"/>
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Typical;
+  happening most often</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>USUAL</t>
+        </is>
+      </c>
+      <c r="C343" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D343" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E343" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="344" ht="21.95" customHeight="1">
-      <c r="C344" s="2" t="n"/>
-      <c r="D344" s="2" t="n"/>
-      <c r="E344" s="2" t="n"/>
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Identical;
+  not different</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>SAME</t>
+        </is>
+      </c>
+      <c r="C344" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D344" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E344" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="345" ht="21.95" customHeight="1">
-      <c r="C345" s="2" t="n"/>
-      <c r="D345" s="2" t="n"/>
-      <c r="E345" s="2" t="n"/>
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>An arm
+  or a leg</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>LIMB</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D345" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E345" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="346" ht="21.95" customHeight="1">
-      <c r="C346" s="2" t="n"/>
-      <c r="D346" s="2" t="n"/>
-      <c r="E346" s="2" t="n"/>
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Forehead,
+  nose, and mouth are on it</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>FACE</t>
+        </is>
+      </c>
+      <c r="C346" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D346" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E346" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="347" ht="21.95" customHeight="1">
-      <c r="C347" s="2" t="n"/>
-      <c r="D347" s="2" t="n"/>
-      <c r="E347" s="2" t="n"/>
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Talk
+  using your voice</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>SPEAK</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D347" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E347" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="348" ht="21.95" customHeight="1">
-      <c r="C348" s="2" t="n"/>
-      <c r="D348" s="2" t="n"/>
-      <c r="E348" s="2" t="n"/>
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>The
+  present day</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>TODAY</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D348" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E348" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="349" ht="21.95" customHeight="1">
-      <c r="C349" s="2" t="n"/>
-      <c r="D349" s="2" t="n"/>
-      <c r="E349" s="2" t="n"/>
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Examine
+  for changes</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="C349" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D349" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E349" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="350" ht="21.95" customHeight="1">
-      <c r="C350" s="2" t="n"/>
-      <c r="D350" s="2" t="n"/>
-      <c r="E350" s="2" t="n"/>
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Organs
+  used for seeing</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>EYES</t>
+        </is>
+      </c>
+      <c r="C350" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D350" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E350" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="351" ht="21.95" customHeight="1">
-      <c r="C351" s="2" t="n"/>
-      <c r="D351" s="2" t="n"/>
-      <c r="E351" s="2" t="n"/>
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Continuing
+  even now</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>STILL</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D351" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E351" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="352" ht="21.95" customHeight="1">
-      <c r="C352" s="2" t="n"/>
-      <c r="D352" s="2" t="n"/>
-      <c r="E352" s="2" t="n"/>
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Recognized
+  from past experience</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>FAMILIAR</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D352" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E352" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="353" ht="21.95" customHeight="1">
-      <c r="C353" s="2" t="n"/>
-      <c r="D353" s="2" t="n"/>
-      <c r="E353" s="2" t="n"/>
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Different
+  from before</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>CHANGED</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D353" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E353" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="354" ht="21.95" customHeight="1">
-      <c r="C354" s="2" t="n"/>
-      <c r="D354" s="2" t="n"/>
-      <c r="E354" s="2" t="n"/>
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Lasting
+  more time than before</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>LONGER</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D354" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E354" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="355" ht="21.95" customHeight="1">
-      <c r="C355" s="2" t="n"/>
-      <c r="D355" s="2" t="n"/>
-      <c r="E355" s="2" t="n"/>
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Time
+  units of 60 seconds</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>MINUTES</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D355" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E355" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="356" ht="21.95" customHeight="1">
-      <c r="C356" s="2" t="n"/>
-      <c r="D356" s="2" t="n"/>
-      <c r="E356" s="2" t="n"/>
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Small
+  facts worth noting</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>DETAILS</t>
+        </is>
+      </c>
+      <c r="C356" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D356" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E356" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="357" ht="21.95" customHeight="1">
-      <c r="C357" s="2" t="n"/>
-      <c r="D357" s="2" t="n"/>
-      <c r="E357" s="2" t="n"/>
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Tell
+  what happened, not why</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>DESCRIBE</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D357" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E357" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="358" ht="21.95" customHeight="1">
-      <c r="C358" s="2" t="n"/>
-      <c r="D358" s="2" t="n"/>
-      <c r="E358" s="2" t="n"/>
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Share
+  symptoms or features</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>OVERLAP</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D358" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E358" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="359" ht="21.95" customHeight="1">
-      <c r="C359" s="2" t="n"/>
-      <c r="D359" s="2" t="n"/>
-      <c r="E359" s="2" t="n"/>
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Reaction
+  to pollen, for example</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>ALLERGY</t>
+        </is>
+      </c>
+      <c r="C359" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D359" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E359" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="360" ht="21.95" customHeight="1">
-      <c r="C360" s="2" t="n"/>
-      <c r="D360" s="2" t="n"/>
-      <c r="E360" s="2" t="n"/>
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Fine
+  powder from flowering plants</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>POLLEN</t>
+        </is>
+      </c>
+      <c r="C360" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D360" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E360" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="361" ht="21.95" customHeight="1">
-      <c r="C361" s="2" t="n"/>
-      <c r="D361" s="2" t="n"/>
-      <c r="E361" s="2" t="n"/>
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Tiny
+  drops of liquid</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>DROPLETS</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D361" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E361" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="362" ht="21.95" customHeight="1">
-      <c r="C362" s="2" t="n"/>
-      <c r="D362" s="2" t="n"/>
-      <c r="E362" s="2" t="n"/>
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>A
+  clinician's hands-on check</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>EXAM</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D362" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E362" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="363" ht="21.95" customHeight="1">
-      <c r="C363" s="2" t="n"/>
-      <c r="D363" s="2" t="n"/>
-      <c r="E363" s="2" t="n"/>
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Routine
+  rather than emergency</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>REGULAR</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D363" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E363" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="364" ht="21.95" customHeight="1">
-      <c r="C364" s="2" t="n"/>
-      <c r="D364" s="2" t="n"/>
-      <c r="E364" s="2" t="n"/>
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Beginning
+  abruptly</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>SUDDEN</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D364" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E364" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="365" ht="21.95" customHeight="1">
-      <c r="C365" s="2" t="n"/>
-      <c r="D365" s="2" t="n"/>
-      <c r="E365" s="2" t="n"/>
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Look for
+  what matches or differs</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>COMPARE</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D365" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E365" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="366" ht="21.95" customHeight="1">
-      <c r="C366" s="2" t="n"/>
-      <c r="D366" s="2" t="n"/>
-      <c r="E366" s="2" t="n"/>
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Already
+  evaluated by a professional</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>ASSESSED</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D366" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E366" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="367" ht="21.95" customHeight="1">
-      <c r="C367" s="2" t="n"/>
-      <c r="D367" s="2" t="n"/>
-      <c r="E367" s="2" t="n"/>
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Needing
+  prompt attention</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>URGENT</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D367" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E367" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="368" ht="21.95" customHeight="1">
-      <c r="C368" s="2" t="n"/>
-      <c r="D368" s="2" t="n"/>
-      <c r="E368" s="2" t="n"/>
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>When
+  something starts or ends</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>TIMING</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D368" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E368" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="369" ht="21.95" customHeight="1">
-      <c r="C369" s="2" t="n"/>
-      <c r="D369" s="2" t="n"/>
-      <c r="E369" s="2" t="n"/>
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Let one
+  diagnosis hide another</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>OVERSHADOW</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D369" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E369" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="370" ht="21.95" customHeight="1">
-      <c r="C370" s="2" t="n"/>
-      <c r="D370" s="2" t="n"/>
-      <c r="E370" s="2" t="n"/>
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>What
+  makes two things unlike</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>DIFFERENCE</t>
+        </is>
+      </c>
+      <c r="C370" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D370" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E370" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="371" ht="21.95" customHeight="1">
-      <c r="C371" s="2" t="n"/>
-      <c r="D371" s="2" t="n"/>
-      <c r="E371" s="2" t="n"/>
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Moving
+  air in and out of lungs</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>BREATHING</t>
+        </is>
+      </c>
+      <c r="C371" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D371" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E371" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="372" ht="21.95" customHeight="1">
-      <c r="C372" s="2" t="n"/>
-      <c r="D372" s="2" t="n"/>
-      <c r="E372" s="2" t="n"/>
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Situation
+  needing help right away</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>EMERGENCY</t>
+        </is>
+      </c>
+      <c r="C372" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D372" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E372" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="373" ht="21.95" customHeight="1">
-      <c r="C373" s="2" t="n"/>
-      <c r="D373" s="2" t="n"/>
-      <c r="E373" s="2" t="n"/>
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Drug
+  prescribed for treatment</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>MEDICATION</t>
+        </is>
+      </c>
+      <c r="C373" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D373" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E373" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="374" ht="21.95" customHeight="1">
-      <c r="C374" s="2" t="n"/>
-      <c r="D374" s="2" t="n"/>
-      <c r="E374" s="2" t="n"/>
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Examine
+  an unexplained problem</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>INVESTIGATE</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D374" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E374" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="375" ht="21.95" customHeight="1">
-      <c r="C375" s="2" t="n"/>
-      <c r="D375" s="2" t="n"/>
-      <c r="E375" s="2" t="n"/>
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>A
+  surprise; not anticipated</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>UNEXPECTED</t>
+        </is>
+      </c>
+      <c r="C375" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D375" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E375" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="376" ht="21.95" customHeight="1">
-      <c r="C376" s="2" t="n"/>
-      <c r="D376" s="2" t="n"/>
-      <c r="E376" s="2" t="n"/>
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Container
+  for carrying essentials</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="C376" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D376" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E376" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="377" ht="21.95" customHeight="1">
-      <c r="C377" s="2" t="n"/>
-      <c r="D377" s="2" t="n"/>
-      <c r="E377" s="2" t="n"/>
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Cover
+  worn over the eyes to block light</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>MASK</t>
+        </is>
+      </c>
+      <c r="C377" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D377" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E377" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="378" ht="21.95" customHeight="1">
-      <c r="C378" s="2" t="n"/>
-      <c r="D378" s="2" t="n"/>
-      <c r="E378" s="2" t="n"/>
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Grab ___
+  beside a bath or toilet</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>BARS</t>
+        </is>
+      </c>
+      <c r="C378" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D378" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E378" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="379" ht="21.95" customHeight="1">
-      <c r="C379" s="2" t="n"/>
-      <c r="D379" s="2" t="n"/>
-      <c r="E379" s="2" t="n"/>
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Light-emitting
+  diode (abbreviation)</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>LED</t>
+        </is>
+      </c>
+      <c r="C379" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D379" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E379" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="380" ht="21.95" customHeight="1">
-      <c r="C380" s="2" t="n"/>
-      <c r="D380" s="2" t="n"/>
-      <c r="E380" s="2" t="n"/>
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Indoor
+  space enclosed by walls</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>ROOM</t>
+        </is>
+      </c>
+      <c r="C380" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D380" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E380" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="381" ht="21.95" customHeight="1">
-      <c r="C381" s="2" t="n"/>
-      <c r="D381" s="2" t="n"/>
-      <c r="E381" s="2" t="n"/>
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Casual
+  word for equipment</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>GEAR</t>
+        </is>
+      </c>
+      <c r="C381" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D381" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E381" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="382" ht="21.95" customHeight="1">
-      <c r="C382" s="2" t="n"/>
-      <c r="D382" s="2" t="n"/>
-      <c r="E382" s="2" t="n"/>
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Pocket
+  device for calls and notes</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>PHONE</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D382" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E382" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="383" ht="21.95" customHeight="1">
-      <c r="C383" s="2" t="n"/>
-      <c r="D383" s="2" t="n"/>
-      <c r="E383" s="2" t="n"/>
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>One page
+  of emergency information</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>SHEET</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D383" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E383" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="384" ht="21.95" customHeight="1">
-      <c r="C384" s="2" t="n"/>
-      <c r="D384" s="2" t="n"/>
-      <c r="E384" s="2" t="n"/>
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Extra;
+  kept just in case</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>SPARE</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D384" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E384" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="385" ht="21.95" customHeight="1">
-      <c r="C385" s="2" t="n"/>
-      <c r="D385" s="2" t="n"/>
-      <c r="E385" s="2" t="n"/>
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Prepared
+  for immediate use</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D385" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E385" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="386" ht="21.95" customHeight="1">
-      <c r="C386" s="2" t="n"/>
-      <c r="D386" s="2" t="n"/>
-      <c r="E386" s="2" t="n"/>
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Bend
+  inward along a hinge</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>FOLD</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D386" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E386" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="387" ht="21.95" customHeight="1">
-      <c r="C387" s="2" t="n"/>
-      <c r="D387" s="2" t="n"/>
-      <c r="E387" s="2" t="n"/>
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Informal
+  word for medications</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>MEDS</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D387" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E387" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="388" ht="21.95" customHeight="1">
-      <c r="C388" s="2" t="n"/>
-      <c r="D388" s="2" t="n"/>
-      <c r="E388" s="2" t="n"/>
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Control
+  for a light's intensity</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>DIMMER</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D388" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E388" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="389" ht="21.95" customHeight="1">
-      <c r="C389" s="2" t="n"/>
-      <c r="D389" s="2" t="n"/>
-      <c r="E389" s="2" t="n"/>
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Bag
+  carried on both shoulders</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>BACKPACK</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D389" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E389" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="390" ht="21.95" customHeight="1">
-      <c r="C390" s="2" t="n"/>
-      <c r="D390" s="2" t="n"/>
-      <c r="E390" s="2" t="n"/>
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Useful
+  items kept on hand</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>SUPPLIES</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D390" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E390" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="391" ht="21.95" customHeight="1">
-      <c r="C391" s="2" t="n"/>
-      <c r="D391" s="2" t="n"/>
-      <c r="E391" s="2" t="n"/>
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Small
+  inserts that reduce noise</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>EARPLUGS</t>
+        </is>
+      </c>
+      <c r="C391" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D391" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E391" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="392" ht="21.95" customHeight="1">
-      <c r="C392" s="2" t="n"/>
-      <c r="D392" s="2" t="n"/>
-      <c r="E392" s="2" t="n"/>
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Considered
+  reliable</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>TRUSTED</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D392" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E392" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="393" ht="21.95" customHeight="1">
-      <c r="C393" s="2" t="n"/>
-      <c r="D393" s="2" t="n"/>
-      <c r="E393" s="2" t="n"/>
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Get
+  organized in advance</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>PREPARE</t>
+        </is>
+      </c>
+      <c r="C393" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D393" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E393" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="394" ht="21.95" customHeight="1">
-      <c r="C394" s="2" t="n"/>
-      <c r="D394" s="2" t="n"/>
-      <c r="E394" s="2" t="n"/>
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Printed
+  sheet of helpful information</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>HANDOUT</t>
+        </is>
+      </c>
+      <c r="C394" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D394" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E394" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="395" ht="21.95" customHeight="1">
-      <c r="C395" s="2" t="n"/>
-      <c r="D395" s="2" t="n"/>
-      <c r="E395" s="2" t="n"/>
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Frame
+  used to assist walking</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>WALKER</t>
+        </is>
+      </c>
+      <c r="C395" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D395" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E395" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="396" ht="21.95" customHeight="1">
-      <c r="C396" s="2" t="n"/>
-      <c r="D396" s="2" t="n"/>
-      <c r="E396" s="2" t="n"/>
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Duplicates
+  of a document</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>COPIES</t>
+        </is>
+      </c>
+      <c r="C396" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D396" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E396" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="397" ht="21.95" customHeight="1">
-      <c r="C397" s="2" t="n"/>
-      <c r="D397" s="2" t="n"/>
-      <c r="E397" s="2" t="n"/>
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Well-known
+  tissue brand</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>KLEENEX</t>
+        </is>
+      </c>
+      <c r="C397" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D397" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E397" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="398" ht="21.95" customHeight="1">
-      <c r="C398" s="2" t="n"/>
-      <c r="D398" s="2" t="n"/>
-      <c r="E398" s="2" t="n"/>
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Person
+  to call in an emergency</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>CONTACT</t>
+        </is>
+      </c>
+      <c r="C398" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D398" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E398" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="399" ht="21.95" customHeight="1">
-      <c r="C399" s="2" t="n"/>
-      <c r="D399" s="2" t="n"/>
-      <c r="E399" s="2" t="n"/>
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Room
+  mainly used for sleeping</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>BEDROOM</t>
+        </is>
+      </c>
+      <c r="C399" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D399" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E399" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="400" ht="21.95" customHeight="1">
-      <c r="C400" s="2" t="n"/>
-      <c r="D400" s="2" t="n"/>
-      <c r="E400" s="2" t="n"/>
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Room
+  surface above your head</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>CEILING</t>
+        </is>
+      </c>
+      <c r="C400" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D400" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E400" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="401" ht="21.95" customHeight="1">
-      <c r="C401" s="2" t="n"/>
-      <c r="D401" s="2" t="n"/>
-      <c r="E401" s="2" t="n"/>
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Absence
+  of light</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>DARKNESS</t>
+        </is>
+      </c>
+      <c r="C401" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D401" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E401" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Ability
+  to move around</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>MOBILITY</t>
+        </is>
+      </c>
+      <c r="C402" t="n">
+        <v>1</v>
+      </c>
+      <c r="D402" t="n">
+        <v>13</v>
+      </c>
+      <c r="E402" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Organize
+  or put in place</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>ARRANGE</t>
+        </is>
+      </c>
+      <c r="C403" t="n">
+        <v>2</v>
+      </c>
+      <c r="D403" t="n">
+        <v>13</v>
+      </c>
+      <c r="E403" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Reduce
+  sound passing through walls</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>SOUNDPROOF</t>
+        </is>
+      </c>
+      <c r="C404" t="n">
+        <v>2</v>
+      </c>
+      <c r="D404" t="n">
+        <v>13</v>
+      </c>
+      <c r="E404" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Intensity
+  of a light</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>BRIGHTNESS</t>
+        </is>
+      </c>
+      <c r="C405" t="n">
+        <v>1</v>
+      </c>
+      <c r="D405" t="n">
+        <v>13</v>
+      </c>
+      <c r="E405" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Directions
+  on what to do</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>INSTRUCTIONS</t>
+        </is>
+      </c>
+      <c r="C406" t="n">
+        <v>1</v>
+      </c>
+      <c r="D406" t="n">
+        <v>13</v>
+      </c>
+      <c r="E406" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Share
+  thoughts or information</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>COMMUNICATE</t>
+        </is>
+      </c>
+      <c r="C407" t="n">
+        <v>1</v>
+      </c>
+      <c r="D407" t="n">
+        <v>13</v>
+      </c>
+      <c r="E407" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Getting
+  ready beforehand</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>PREPARATION</t>
+        </is>
+      </c>
+      <c r="C408" t="n">
+        <v>1</v>
+      </c>
+      <c r="D408" t="n">
+        <v>13</v>
+      </c>
+      <c r="E408" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Practical
+  change to fit a need</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>ADAPTATION</t>
+        </is>
+      </c>
+      <c r="C409" t="n">
+        <v>1</v>
+      </c>
+      <c r="D409" t="n">
+        <v>13</v>
+      </c>
+      <c r="E409" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Easy to
+  reach or use</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>ACCESSIBLE</t>
+        </is>
+      </c>
+      <c r="C410" t="n">
+        <v>2</v>
+      </c>
+      <c r="D410" t="n">
+        <v>13</v>
+      </c>
+      <c r="E410" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Public
+  green space for a stroll</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>PARK</t>
+        </is>
+      </c>
+      <c r="C411" t="n">
+        <v>2</v>
+      </c>
+      <c r="D411" t="n">
+        <v>14</v>
+      </c>
+      <c r="E411" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Path
+  through a park or forest</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>TRAIL</t>
+        </is>
+      </c>
+      <c r="C412" t="n">
+        <v>1</v>
+      </c>
+      <c r="D412" t="n">
+        <v>14</v>
+      </c>
+      <c r="E412" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Place to
+  sit</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>SEAT</t>
+        </is>
+      </c>
+      <c r="C413" t="n">
+        <v>1</v>
+      </c>
+      <c r="D413" t="n">
+        <v>14</v>
+      </c>
+      <c r="E413" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Path
+  taken to a destination</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>ROUTE</t>
+        </is>
+      </c>
+      <c r="C414" t="n">
+        <v>1</v>
+      </c>
+      <c r="D414" t="n">
+        <v>14</v>
+      </c>
+      <c r="E414" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Way out</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>EXIT</t>
+        </is>
+      </c>
+      <c r="C415" t="n">
+        <v>2</v>
+      </c>
+      <c r="D415" t="n">
+        <v>14</v>
+      </c>
+      <c r="E415" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Unplanned
+  drop to the ground</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>FALL</t>
+        </is>
+      </c>
+      <c r="C416" t="n">
+        <v>1</v>
+      </c>
+      <c r="D416" t="n">
+        <v>14</v>
+      </c>
+      <c r="E416" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>In pain</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>HURT</t>
+        </is>
+      </c>
+      <c r="C417" t="n">
+        <v>2</v>
+      </c>
+      <c r="D417" t="n">
+        <v>14</v>
+      </c>
+      <c r="E417" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Cease an
+  unsafe action</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>STOP</t>
+        </is>
+      </c>
+      <c r="C418" t="n">
+        <v>2</v>
+      </c>
+      <c r="D418" t="n">
+        <v>14</v>
+      </c>
+      <c r="E418" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>After
+  some time has passed</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>LATER</t>
+        </is>
+      </c>
+      <c r="C419" t="n">
+        <v>2</v>
+      </c>
+      <c r="D419" t="n">
+        <v>14</v>
+      </c>
+      <c r="E419" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>In
+  advance; before leaving</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>AHEAD</t>
+        </is>
+      </c>
+      <c r="C420" t="n">
+        <v>2</v>
+      </c>
+      <c r="D420" t="n">
+        <v>14</v>
+      </c>
+      <c r="E420" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Raise
+  off the ground</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>LIFT</t>
+        </is>
+      </c>
+      <c r="C421" t="n">
+        <v>3</v>
+      </c>
+      <c r="D421" t="n">
+        <v>14</v>
+      </c>
+      <c r="E421" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Travel
+  on foot</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>WALK</t>
+        </is>
+      </c>
+      <c r="C422" t="n">
+        <v>2</v>
+      </c>
+      <c r="D422" t="n">
+        <v>14</v>
+      </c>
+      <c r="E422" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Possible
+  sources of harm</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>HAZARDS</t>
+        </is>
+      </c>
+      <c r="C423" t="n">
+        <v>1</v>
+      </c>
+      <c r="D423" t="n">
+        <v>14</v>
+      </c>
+      <c r="E423" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Keep
+  safe from danger</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>PROTECT</t>
+        </is>
+      </c>
+      <c r="C424" t="n">
+        <v>1</v>
+      </c>
+      <c r="D424" t="n">
+        <v>14</v>
+      </c>
+      <c r="E424" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Alternative
+  when the first plan fails</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>BACKUP</t>
+        </is>
+      </c>
+      <c r="C425" t="n">
+        <v>2</v>
+      </c>
+      <c r="D425" t="n">
+        <v>14</v>
+      </c>
+      <c r="E425" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Physically
+  harmed in an accident</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>INJURED</t>
+        </is>
+      </c>
+      <c r="C426" t="n">
+        <v>1</v>
+      </c>
+      <c r="D426" t="n">
+        <v>14</v>
+      </c>
+      <c r="E426" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Look
+  over once more</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>RECHECK</t>
+        </is>
+      </c>
+      <c r="C427" t="n">
+        <v>2</v>
+      </c>
+      <c r="D427" t="n">
+        <v>14</v>
+      </c>
+      <c r="E427" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>React to
+  what happens</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>RESPOND</t>
+        </is>
+      </c>
+      <c r="C428" t="n">
+        <v>2</v>
+      </c>
+      <c r="D428" t="n">
+        <v>14</v>
+      </c>
+      <c r="E428" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Boundaries
+  of what someone can manage</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>LIMITS</t>
+        </is>
+      </c>
+      <c r="C429" t="n">
+        <v>1</v>
+      </c>
+      <c r="D429" t="n">
+        <v>14</v>
+      </c>
+      <c r="E429" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Ready
+  for what may happen</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>PREPARED</t>
+        </is>
+      </c>
+      <c r="C430" t="n">
+        <v>1</v>
+      </c>
+      <c r="D430" t="n">
+        <v>14</v>
+      </c>
+      <c r="E430" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Obstacles
+  blocking access</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>BARRIERS</t>
+        </is>
+      </c>
+      <c r="C431" t="n">
+        <v>2</v>
+      </c>
+      <c r="D431" t="n">
+        <v>14</v>
+      </c>
+      <c r="E431" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Available
+  alternatives</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>OPTIONS</t>
+        </is>
+      </c>
+      <c r="C432" t="n">
+        <v>2</v>
+      </c>
+      <c r="D432" t="n">
+        <v>14</v>
+      </c>
+      <c r="E432" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Consider
+  a different approach</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>RETHINK</t>
+        </is>
+      </c>
+      <c r="C433" t="n">
+        <v>2</v>
+      </c>
+      <c r="D433" t="n">
+        <v>14</v>
+      </c>
+      <c r="E433" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Staying
+  until something happens</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>WAITING</t>
+        </is>
+      </c>
+      <c r="C434" t="n">
+        <v>3</v>
+      </c>
+      <c r="D434" t="n">
+        <v>14</v>
+      </c>
+      <c r="E434" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Steps
+  connecting different floors</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>STAIRS</t>
+        </is>
+      </c>
+      <c r="C435" t="n">
+        <v>2</v>
+      </c>
+      <c r="D435" t="n">
+        <v>14</v>
+      </c>
+      <c r="E435" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Space
+  between two places</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>DISTANCE</t>
+        </is>
+      </c>
+      <c r="C436" t="n">
+        <v>3</v>
+      </c>
+      <c r="D436" t="n">
+        <v>14</v>
+      </c>
+      <c r="E436" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Tailored
+  to one individual</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>PERSONAL</t>
+        </is>
+      </c>
+      <c r="C437" t="n">
+        <v>2</v>
+      </c>
+      <c r="D437" t="n">
+        <v>14</v>
+      </c>
+      <c r="E437" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Professional
+  treatment or rehabilitation</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>THERAPY</t>
+        </is>
+      </c>
+      <c r="C438" t="n">
+        <v>2</v>
+      </c>
+      <c r="D438" t="n">
+        <v>14</v>
+      </c>
+      <c r="E438" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Painful
+  sensitivity to ordinary sounds</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>HYPERACUSIS</t>
+        </is>
+      </c>
+      <c r="C439" t="n">
+        <v>1</v>
+      </c>
+      <c r="D439" t="n">
+        <v>14</v>
+      </c>
+      <c r="E439" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Back-and-forth
+  discussion</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>CONVERSATION</t>
+        </is>
+      </c>
+      <c r="C440" t="n">
+        <v>1</v>
+      </c>
+      <c r="D440" t="n">
+        <v>14</v>
+      </c>
+      <c r="E440" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Not
+  previously known</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>UNFAMILIAR</t>
+        </is>
+      </c>
+      <c r="C441" t="n">
+        <v>2</v>
+      </c>
+      <c r="D441" t="n">
+        <v>14</v>
+      </c>
+      <c r="E441" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Entire
+  stair structure between floors</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>STAIRCASE</t>
+        </is>
+      </c>
+      <c r="C442" t="n">
+        <v>2</v>
+      </c>
+      <c r="D442" t="n">
+        <v>14</v>
+      </c>
+      <c r="E442" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Health
+  and comfort</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>WELLBEING</t>
+        </is>
+      </c>
+      <c r="C443" t="n">
+        <v>1</v>
+      </c>
+      <c r="D443" t="n">
+        <v>14</v>
+      </c>
+      <c r="E443" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Moving
+  to a higher level of care</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>ESCALATION</t>
+        </is>
+      </c>
+      <c r="C444" t="n">
+        <v>1</v>
+      </c>
+      <c r="D444" t="n">
+        <v>14</v>
+      </c>
+      <c r="E444" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Able to
+  change when needed</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>ADJUSTABLE</t>
+        </is>
+      </c>
+      <c r="C445" t="n">
+        <v>1</v>
+      </c>
+      <c r="D445" t="n">
+        <v>14</v>
+      </c>
+      <c r="E445" t="n">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Save crossword workbook after interrupted session
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -370,7 +370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E445"/>
+  <dimension ref="A1:E519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="70.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9732,6 +9732,1633 @@
       </c>
       <c r="E445" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Brief
+  signal that directs attention or guides an action</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>CUE</t>
+        </is>
+      </c>
+      <c r="C446" t="n">
+        <v>1</v>
+      </c>
+      <c r="D446" t="n">
+        <v>15</v>
+      </c>
+      <c r="E446" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Something
+  that helps someone remember what comes next</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>HINT</t>
+        </is>
+      </c>
+      <c r="C447" t="n">
+        <v>2</v>
+      </c>
+      <c r="D447" t="n">
+        <v>15</v>
+      </c>
+      <c r="E447" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Notice a
+  sound with your ears</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>HEAR</t>
+        </is>
+      </c>
+      <c r="C448" t="n">
+        <v>2</v>
+      </c>
+      <c r="D448" t="n">
+        <v>15</v>
+      </c>
+      <c r="E448" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Make
+  meaning from written words</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="C449" t="n">
+        <v>3</v>
+      </c>
+      <c r="D449" t="n">
+        <v>15</v>
+      </c>
+      <c r="E449" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Enter
+  words using a keyboard</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>TYPE</t>
+        </is>
+      </c>
+      <c r="C450" t="n">
+        <v>3</v>
+      </c>
+      <c r="D450" t="n">
+        <v>15</v>
+      </c>
+      <c r="E450" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Short
+  stop before continuing an activity</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>PAUSE</t>
+        </is>
+      </c>
+      <c r="C451" t="n">
+        <v>2</v>
+      </c>
+      <c r="D451" t="n">
+        <v>15</v>
+      </c>
+      <c r="E451" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Sound
+  that may interrupt concentration</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>RING</t>
+        </is>
+      </c>
+      <c r="C452" t="n">
+        <v>3</v>
+      </c>
+      <c r="D452" t="n">
+        <v>15</v>
+      </c>
+      <c r="E452" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Pay
+  attention to what another person is saying</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>LISTEN</t>
+        </is>
+      </c>
+      <c r="C453" t="n">
+        <v>2</v>
+      </c>
+      <c r="D453" t="n">
+        <v>15</v>
+      </c>
+      <c r="E453" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Separate
+  important information from competing input</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>FILTER</t>
+        </is>
+      </c>
+      <c r="C454" t="n">
+        <v>1</v>
+      </c>
+      <c r="D454" t="n">
+        <v>15</v>
+      </c>
+      <c r="E454" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Choose
+  one item from several possibilities</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>SELECT</t>
+        </is>
+      </c>
+      <c r="C455" t="n">
+        <v>2</v>
+      </c>
+      <c r="D455" t="n">
+        <v>15</v>
+      </c>
+      <c r="E455" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Toward
+  your own thoughts or body sensations</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="C456" t="n">
+        <v>1</v>
+      </c>
+      <c r="D456" t="n">
+        <v>15</v>
+      </c>
+      <c r="E456" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Toward
+  people or events around you</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>OUTWARD</t>
+        </is>
+      </c>
+      <c r="C457" t="n">
+        <v>1</v>
+      </c>
+      <c r="D457" t="n">
+        <v>15</v>
+      </c>
+      <c r="E457" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Attention
+  shared between two activities</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>DIVIDED</t>
+        </is>
+      </c>
+      <c r="C458" t="n">
+        <v>1</v>
+      </c>
+      <c r="D458" t="n">
+        <v>15</v>
+      </c>
+      <c r="E458" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Stays on
+  an activity over time</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>SUSTAINED</t>
+        </is>
+      </c>
+      <c r="C459" t="n">
+        <v>1</v>
+      </c>
+      <c r="D459" t="n">
+        <v>15</v>
+      </c>
+      <c r="E459" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Follow
+  one person speaking: _________ attention.</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>SELECTIVE</t>
+        </is>
+      </c>
+      <c r="C460" t="n">
+        <v>1</v>
+      </c>
+      <c r="D460" t="n">
+        <v>15</v>
+      </c>
+      <c r="E460" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Change
+  from one task to another</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>SWITCH</t>
+        </is>
+      </c>
+      <c r="C461" t="n">
+        <v>1</v>
+      </c>
+      <c r="D461" t="n">
+        <v>15</v>
+      </c>
+      <c r="E461" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Turn
+  your attention toward a new sound or event</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>ORIENT</t>
+        </is>
+      </c>
+      <c r="C462" t="n">
+        <v>2</v>
+      </c>
+      <c r="D462" t="n">
+        <v>15</v>
+      </c>
+      <c r="E462" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Bring
+  attention back after it has wandered</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>REFOCUS</t>
+        </is>
+      </c>
+      <c r="C463" t="n">
+        <v>1</v>
+      </c>
+      <c r="D463" t="n">
+        <v>15</v>
+      </c>
+      <c r="E463" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Continue
+  a task after an interruption</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>RESUME</t>
+        </is>
+      </c>
+      <c r="C464" t="n">
+        <v>2</v>
+      </c>
+      <c r="D464" t="n">
+        <v>15</v>
+      </c>
+      <c r="E464" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Short
+  reminder that helps someone carry on</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>PROMPT</t>
+        </is>
+      </c>
+      <c r="C465" t="n">
+        <v>2</v>
+      </c>
+      <c r="D465" t="n">
+        <v>15</v>
+      </c>
+      <c r="E465" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>More
+  information or demands than someone can comfortably handle</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>OVERLOAD</t>
+        </is>
+      </c>
+      <c r="C466" t="n">
+        <v>1</v>
+      </c>
+      <c r="D466" t="n">
+        <v>15</v>
+      </c>
+      <c r="E466" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Bring a
+  fact or instruction back to mind</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>REMEMBER</t>
+        </is>
+      </c>
+      <c r="C467" t="n">
+        <v>2</v>
+      </c>
+      <c r="D467" t="n">
+        <v>15</v>
+      </c>
+      <c r="E467" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Reduce
+  unnecessary steps</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>SIMPLIFY</t>
+        </is>
+      </c>
+      <c r="C468" t="n">
+        <v>2</v>
+      </c>
+      <c r="D468" t="n">
+        <v>15</v>
+      </c>
+      <c r="E468" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Demands
+  pulling for a person's attention</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>COMPETING</t>
+        </is>
+      </c>
+      <c r="C469" t="n">
+        <v>1</v>
+      </c>
+      <c r="D469" t="n">
+        <v>15</v>
+      </c>
+      <c r="E469" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Information
+  that matters to the task at hand</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>RELEVANCE</t>
+        </is>
+      </c>
+      <c r="C470" t="n">
+        <v>2</v>
+      </c>
+      <c r="D470" t="n">
+        <v>15</v>
+      </c>
+      <c r="E470" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Less
+  prominent details</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>BACKGROUND</t>
+        </is>
+      </c>
+      <c r="C471" t="n">
+        <v>3</v>
+      </c>
+      <c r="D471" t="n">
+        <v>15</v>
+      </c>
+      <c r="E471" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>A hint
+  of where to return to a paused task</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>BREADCRUMB</t>
+        </is>
+      </c>
+      <c r="C472" t="n">
+        <v>1</v>
+      </c>
+      <c r="D472" t="n">
+        <v>15</v>
+      </c>
+      <c r="E472" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>draws attention away</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>DISTRACTION</t>
+        </is>
+      </c>
+      <c r="C473" t="n">
+        <v>1</v>
+      </c>
+      <c r="D473" t="n">
+        <v>15</v>
+      </c>
+      <c r="E473" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Breaks a
+  person's concentration</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>INTERRUPTION</t>
+        </is>
+      </c>
+      <c r="C474" t="n">
+        <v>1</v>
+      </c>
+      <c r="D474" t="n">
+        <v>15</v>
+      </c>
+      <c r="E474" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Focus
+  attention</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>CONCENTRATE</t>
+        </is>
+      </c>
+      <c r="C475" t="n">
+        <v>1</v>
+      </c>
+      <c r="D475" t="n">
+        <v>15</v>
+      </c>
+      <c r="E475" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Put the
+  most important demand first</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>PRIORITIZE</t>
+        </is>
+      </c>
+      <c r="C476" t="n">
+        <v>1</v>
+      </c>
+      <c r="D476" t="n">
+        <v>15</v>
+      </c>
+      <c r="E476" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>How
+  firmly a hand holds an object</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>GRIP</t>
+        </is>
+      </c>
+      <c r="C477" t="n">
+        <v>1</v>
+      </c>
+      <c r="D477" t="n">
+        <v>16</v>
+      </c>
+      <c r="E477" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Extend
+  an arm toward an object</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>REACH</t>
+        </is>
+      </c>
+      <c r="C478" t="n">
+        <v>1</v>
+      </c>
+      <c r="D478" t="n">
+        <v>16</v>
+      </c>
+      <c r="E478" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Joint
+  between the forearm and the hand</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>WRIST</t>
+        </is>
+      </c>
+      <c r="C479" t="n">
+        <v>3</v>
+      </c>
+      <c r="D479" t="n">
+        <v>16</v>
+      </c>
+      <c r="E479" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Ability
+  developed through learning and repeated use</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>SKILL</t>
+        </is>
+      </c>
+      <c r="C480" t="n">
+        <v>1</v>
+      </c>
+      <c r="D480" t="n">
+        <v>16</v>
+      </c>
+      <c r="E480" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Familiar
+  routine that may need little step-by-step thought</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>HABIT</t>
+        </is>
+      </c>
+      <c r="C481" t="n">
+        <v>2</v>
+      </c>
+      <c r="D481" t="n">
+        <v>16</v>
+      </c>
+      <c r="E481" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Close
+  the hand around an object to hold it</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>GRASP</t>
+        </is>
+      </c>
+      <c r="C482" t="n">
+        <v>2</v>
+      </c>
+      <c r="D482" t="n">
+        <v>16</v>
+      </c>
+      <c r="E482" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Body
+  tissue that contracts to move a joint</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>MUSCLE</t>
+        </is>
+      </c>
+      <c r="C483" t="n">
+        <v>3</v>
+      </c>
+      <c r="D483" t="n">
+        <v>16</v>
+      </c>
+      <c r="E483" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Let go
+  of something after holding it</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>RELEASE</t>
+        </is>
+      </c>
+      <c r="C484" t="n">
+        <v>2</v>
+      </c>
+      <c r="D484" t="n">
+        <v>16</v>
+      </c>
+      <c r="E484" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>How the
+  body is positioned during an activity</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>POSTURE</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>3</v>
+      </c>
+      <c r="D485" t="n">
+        <v>16</v>
+      </c>
+      <c r="E485" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Work on
+  improving an existing movement through guided practice</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>RETRAIN</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>1</v>
+      </c>
+      <c r="D486" t="n">
+        <v>16</v>
+      </c>
+      <c r="E486" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Smooth,
+  connected performance of a familiar action</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>FLUENCY</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>1</v>
+      </c>
+      <c r="D487" t="n">
+        <v>16</v>
+      </c>
+      <c r="E487" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Ordered
+  series of actions making up a learned skill</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>SEQUENCE</t>
+        </is>
+      </c>
+      <c r="C488" t="n">
+        <v>1</v>
+      </c>
+      <c r="D488" t="n">
+        <v>16</v>
+      </c>
+      <c r="E488" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Everyday
+  activity of putting on clothes</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>DRESSING</t>
+        </is>
+      </c>
+      <c r="C489" t="n">
+        <v>1</v>
+      </c>
+      <c r="D489" t="n">
+        <v>16</v>
+      </c>
+      <c r="E489" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Move
+  from one surface to another, such as bed to chair</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>TRANSFER</t>
+        </is>
+      </c>
+      <c r="C490" t="n">
+        <v>1</v>
+      </c>
+      <c r="D490" t="n">
+        <v>16</v>
+      </c>
+      <c r="E490" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Joint
+  connecting the upper arm to the body</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>SHOULDER</t>
+        </is>
+      </c>
+      <c r="C491" t="n">
+        <v>3</v>
+      </c>
+      <c r="D491" t="n">
+        <v>16</v>
+      </c>
+      <c r="E491" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Practise
+  an action in preparation for using it</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>REHEARSE</t>
+        </is>
+      </c>
+      <c r="C492" t="n">
+        <v>2</v>
+      </c>
+      <c r="D492" t="n">
+        <v>16</v>
+      </c>
+      <c r="E492" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Type of
+  memory for events a person has experienced</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>EPISODIC</t>
+        </is>
+      </c>
+      <c r="C493" t="n">
+        <v>3</v>
+      </c>
+      <c r="D493" t="n">
+        <v>16</v>
+      </c>
+      <c r="E493" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Describes
+  an intentional effort to move on command</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>VOLUNTARY</t>
+        </is>
+      </c>
+      <c r="C494" t="n">
+        <v>1</v>
+      </c>
+      <c r="D494" t="n">
+        <v>16</v>
+      </c>
+      <c r="E494" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Ability
+  to keep an activity going over time</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>ENDURANCE</t>
+        </is>
+      </c>
+      <c r="C495" t="n">
+        <v>1</v>
+      </c>
+      <c r="D495" t="n">
+        <v>16</v>
+      </c>
+      <c r="E495" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Help
+  that may still be needed even when some movement occurs</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>ASSISTANCE</t>
+        </is>
+      </c>
+      <c r="C496" t="n">
+        <v>1</v>
+      </c>
+      <c r="D496" t="n">
+        <v>16</v>
+      </c>
+      <c r="E496" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Brain
+  structure involved in fine-tuning movement and motor learning</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>CEREBELLUM</t>
+        </is>
+      </c>
+      <c r="C497" t="n">
+        <v>2</v>
+      </c>
+      <c r="D497" t="n">
+        <v>16</v>
+      </c>
+      <c r="E497" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Type of
+  memory that supports learned skills such as typing</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>PROCEDURAL</t>
+        </is>
+      </c>
+      <c r="C498" t="n">
+        <v>1</v>
+      </c>
+      <c r="D498" t="n">
+        <v>16</v>
+      </c>
+      <c r="E498" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Make
+  several muscles or joints work together on an action</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>COORDINATE</t>
+        </is>
+      </c>
+      <c r="C499" t="n">
+        <v>1</v>
+      </c>
+      <c r="D499" t="n">
+        <v>16</v>
+      </c>
+      <c r="E499" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Describes
+  an action that can be performed again in similar conditions</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>REPEATABLE</t>
+        </is>
+      </c>
+      <c r="C500" t="n">
+        <v>1</v>
+      </c>
+      <c r="D500" t="n">
+        <v>16</v>
+      </c>
+      <c r="E500" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Toward a
+  chosen target</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>AIM</t>
+        </is>
+      </c>
+      <c r="C501" t="n">
+        <v>1</v>
+      </c>
+      <c r="D501" t="n">
+        <v>17</v>
+      </c>
+      <c r="E501" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Can
+  provide movement timing</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>BEAT</t>
+        </is>
+      </c>
+      <c r="C502" t="n">
+        <v>3</v>
+      </c>
+      <c r="D502" t="n">
+        <v>17</v>
+      </c>
+      <c r="E502" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Store
+  your books here.</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>SHELF</t>
+        </is>
+      </c>
+      <c r="C503" t="n">
+        <v>3</v>
+      </c>
+      <c r="D503" t="n">
+        <v>17</v>
+      </c>
+      <c r="E503" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Firmly
+  in the hand.</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="C504" t="n">
+        <v>3</v>
+      </c>
+      <c r="D504" t="n">
+        <v>17</v>
+      </c>
+      <c r="E504" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Put an
+  object where it belongs</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>PLACE</t>
+        </is>
+      </c>
+      <c r="C505" t="n">
+        <v>3</v>
+      </c>
+      <c r="D505" t="n">
+        <v>17</v>
+      </c>
+      <c r="E505" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Physical
+  item whose shape and weight affect how it is handled</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>OBJECT</t>
+        </is>
+      </c>
+      <c r="C506" t="n">
+        <v>3</v>
+      </c>
+      <c r="D506" t="n">
+        <v>17</v>
+      </c>
+      <c r="E506" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>How
+  heavy an object is</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>WEIGHT</t>
+        </is>
+      </c>
+      <c r="C507" t="n">
+        <v>1</v>
+      </c>
+      <c r="D507" t="n">
+        <v>17</v>
+      </c>
+      <c r="E507" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Force
+  that makes lifting different from sliding on a table</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>GRAVITY</t>
+        </is>
+      </c>
+      <c r="C508" t="n">
+        <v>1</v>
+      </c>
+      <c r="D508" t="n">
+        <v>17</v>
+      </c>
+      <c r="E508" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Task,
+  surroundings and available help around an activity</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>CONTEXT</t>
+        </is>
+      </c>
+      <c r="C509" t="n">
+        <v>1</v>
+      </c>
+      <c r="D509" t="n">
+        <v>17</v>
+      </c>
+      <c r="E509" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>This
+  matters alongside task completion</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>COMFORT</t>
+        </is>
+      </c>
+      <c r="C510" t="n">
+        <v>2</v>
+      </c>
+      <c r="D510" t="n">
+        <v>17</v>
+      </c>
+      <c r="E510" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Doing
+  two things at once</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>DUALTASK</t>
+        </is>
+      </c>
+      <c r="C511" t="n">
+        <v>1</v>
+      </c>
+      <c r="D511" t="n">
+        <v>17</v>
+      </c>
+      <c r="E511" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Ffocus
+  directed toward a movement's destination.</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>EXTERNAL</t>
+        </is>
+      </c>
+      <c r="C512" t="n">
+        <v>1</v>
+      </c>
+      <c r="D512" t="n">
+        <v>17</v>
+      </c>
+      <c r="E512" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Focus
+  directed toward the body's own movements</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>INTERNAL</t>
+        </is>
+      </c>
+      <c r="C513" t="n">
+        <v>1</v>
+      </c>
+      <c r="D513" t="n">
+        <v>17</v>
+      </c>
+      <c r="E513" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Information
+  about how an activity went</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>FEEDBACK</t>
+        </is>
+      </c>
+      <c r="C514" t="n">
+        <v>1</v>
+      </c>
+      <c r="D514" t="n">
+        <v>17</v>
+      </c>
+      <c r="E514" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Using a
+  helpful strategy outside the setting where it was learned</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>CARRYOVER</t>
+        </is>
+      </c>
+      <c r="C515" t="n">
+        <v>1</v>
+      </c>
+      <c r="D515" t="n">
+        <v>17</v>
+      </c>
+      <c r="E515" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Move
+  items around to make a task easier</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>REARRANGE</t>
+        </is>
+      </c>
+      <c r="C516" t="n">
+        <v>1</v>
+      </c>
+      <c r="D516" t="n">
+        <v>17</v>
+      </c>
+      <c r="E516" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Qualified
+  professional who can help choose suitable rehabilitation tasks</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>THERAPIST</t>
+        </is>
+      </c>
+      <c r="C517" t="n">
+        <v>3</v>
+      </c>
+      <c r="D517" t="n">
+        <v>17</v>
+      </c>
+      <c r="E517" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>A person
+  whose preferences and responses may differ from others</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>INDIVIDUAL</t>
+        </is>
+      </c>
+      <c r="C518" t="n">
+        <v>2</v>
+      </c>
+      <c r="D518" t="n">
+        <v>17</v>
+      </c>
+      <c r="E518" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Description
+  of what someone noticed</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>OBSERVATION</t>
+        </is>
+      </c>
+      <c r="C519" t="n">
+        <v>1</v>
+      </c>
+      <c r="D519" t="n">
+        <v>17</v>
+      </c>
+      <c r="E519" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recover saved crossword workbook (#195)
Preserves workbook edits saved before the Codespace stopped.
</commit_message>
<xml_diff>
--- a/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
+++ b/tools/puzzles/FND_Crossword_Question_Bank_Template.xlsx
@@ -370,7 +370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E445"/>
+  <dimension ref="A1:E519"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="70.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9732,6 +9732,1633 @@
       </c>
       <c r="E445" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Brief
+  signal that directs attention or guides an action</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>CUE</t>
+        </is>
+      </c>
+      <c r="C446" t="n">
+        <v>1</v>
+      </c>
+      <c r="D446" t="n">
+        <v>15</v>
+      </c>
+      <c r="E446" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Something
+  that helps someone remember what comes next</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>HINT</t>
+        </is>
+      </c>
+      <c r="C447" t="n">
+        <v>2</v>
+      </c>
+      <c r="D447" t="n">
+        <v>15</v>
+      </c>
+      <c r="E447" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Notice a
+  sound with your ears</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>HEAR</t>
+        </is>
+      </c>
+      <c r="C448" t="n">
+        <v>2</v>
+      </c>
+      <c r="D448" t="n">
+        <v>15</v>
+      </c>
+      <c r="E448" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Make
+  meaning from written words</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="C449" t="n">
+        <v>3</v>
+      </c>
+      <c r="D449" t="n">
+        <v>15</v>
+      </c>
+      <c r="E449" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Enter
+  words using a keyboard</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>TYPE</t>
+        </is>
+      </c>
+      <c r="C450" t="n">
+        <v>3</v>
+      </c>
+      <c r="D450" t="n">
+        <v>15</v>
+      </c>
+      <c r="E450" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Short
+  stop before continuing an activity</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>PAUSE</t>
+        </is>
+      </c>
+      <c r="C451" t="n">
+        <v>2</v>
+      </c>
+      <c r="D451" t="n">
+        <v>15</v>
+      </c>
+      <c r="E451" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Sound
+  that may interrupt concentration</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>RING</t>
+        </is>
+      </c>
+      <c r="C452" t="n">
+        <v>3</v>
+      </c>
+      <c r="D452" t="n">
+        <v>15</v>
+      </c>
+      <c r="E452" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Pay
+  attention to what another person is saying</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>LISTEN</t>
+        </is>
+      </c>
+      <c r="C453" t="n">
+        <v>2</v>
+      </c>
+      <c r="D453" t="n">
+        <v>15</v>
+      </c>
+      <c r="E453" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Separate
+  important information from competing input</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>FILTER</t>
+        </is>
+      </c>
+      <c r="C454" t="n">
+        <v>1</v>
+      </c>
+      <c r="D454" t="n">
+        <v>15</v>
+      </c>
+      <c r="E454" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Choose
+  one item from several possibilities</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>SELECT</t>
+        </is>
+      </c>
+      <c r="C455" t="n">
+        <v>2</v>
+      </c>
+      <c r="D455" t="n">
+        <v>15</v>
+      </c>
+      <c r="E455" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Toward
+  your own thoughts or body sensations</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>INWARD</t>
+        </is>
+      </c>
+      <c r="C456" t="n">
+        <v>1</v>
+      </c>
+      <c r="D456" t="n">
+        <v>15</v>
+      </c>
+      <c r="E456" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Toward
+  people or events around you</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>OUTWARD</t>
+        </is>
+      </c>
+      <c r="C457" t="n">
+        <v>1</v>
+      </c>
+      <c r="D457" t="n">
+        <v>15</v>
+      </c>
+      <c r="E457" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Attention
+  shared between two activities</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>DIVIDED</t>
+        </is>
+      </c>
+      <c r="C458" t="n">
+        <v>1</v>
+      </c>
+      <c r="D458" t="n">
+        <v>15</v>
+      </c>
+      <c r="E458" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Stays on
+  an activity over time</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>SUSTAINED</t>
+        </is>
+      </c>
+      <c r="C459" t="n">
+        <v>1</v>
+      </c>
+      <c r="D459" t="n">
+        <v>15</v>
+      </c>
+      <c r="E459" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Follow
+  one person speaking: _________ attention.</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>SELECTIVE</t>
+        </is>
+      </c>
+      <c r="C460" t="n">
+        <v>1</v>
+      </c>
+      <c r="D460" t="n">
+        <v>15</v>
+      </c>
+      <c r="E460" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Change
+  from one task to another</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>SWITCH</t>
+        </is>
+      </c>
+      <c r="C461" t="n">
+        <v>1</v>
+      </c>
+      <c r="D461" t="n">
+        <v>15</v>
+      </c>
+      <c r="E461" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Turn
+  your attention toward a new sound or event</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>ORIENT</t>
+        </is>
+      </c>
+      <c r="C462" t="n">
+        <v>2</v>
+      </c>
+      <c r="D462" t="n">
+        <v>15</v>
+      </c>
+      <c r="E462" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Bring
+  attention back after it has wandered</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>REFOCUS</t>
+        </is>
+      </c>
+      <c r="C463" t="n">
+        <v>1</v>
+      </c>
+      <c r="D463" t="n">
+        <v>15</v>
+      </c>
+      <c r="E463" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Continue
+  a task after an interruption</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>RESUME</t>
+        </is>
+      </c>
+      <c r="C464" t="n">
+        <v>2</v>
+      </c>
+      <c r="D464" t="n">
+        <v>15</v>
+      </c>
+      <c r="E464" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Short
+  reminder that helps someone carry on</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>PROMPT</t>
+        </is>
+      </c>
+      <c r="C465" t="n">
+        <v>2</v>
+      </c>
+      <c r="D465" t="n">
+        <v>15</v>
+      </c>
+      <c r="E465" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>More
+  information or demands than someone can comfortably handle</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>OVERLOAD</t>
+        </is>
+      </c>
+      <c r="C466" t="n">
+        <v>1</v>
+      </c>
+      <c r="D466" t="n">
+        <v>15</v>
+      </c>
+      <c r="E466" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Bring a
+  fact or instruction back to mind</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>REMEMBER</t>
+        </is>
+      </c>
+      <c r="C467" t="n">
+        <v>2</v>
+      </c>
+      <c r="D467" t="n">
+        <v>15</v>
+      </c>
+      <c r="E467" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Reduce
+  unnecessary steps</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>SIMPLIFY</t>
+        </is>
+      </c>
+      <c r="C468" t="n">
+        <v>2</v>
+      </c>
+      <c r="D468" t="n">
+        <v>15</v>
+      </c>
+      <c r="E468" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Demands
+  pulling for a person's attention</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>COMPETING</t>
+        </is>
+      </c>
+      <c r="C469" t="n">
+        <v>1</v>
+      </c>
+      <c r="D469" t="n">
+        <v>15</v>
+      </c>
+      <c r="E469" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Information
+  that matters to the task at hand</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>RELEVANCE</t>
+        </is>
+      </c>
+      <c r="C470" t="n">
+        <v>2</v>
+      </c>
+      <c r="D470" t="n">
+        <v>15</v>
+      </c>
+      <c r="E470" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Less
+  prominent details</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>BACKGROUND</t>
+        </is>
+      </c>
+      <c r="C471" t="n">
+        <v>3</v>
+      </c>
+      <c r="D471" t="n">
+        <v>15</v>
+      </c>
+      <c r="E471" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>A hint
+  of where to return to a paused task</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>BREADCRUMB</t>
+        </is>
+      </c>
+      <c r="C472" t="n">
+        <v>1</v>
+      </c>
+      <c r="D472" t="n">
+        <v>15</v>
+      </c>
+      <c r="E472" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>draws attention away</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>DISTRACTION</t>
+        </is>
+      </c>
+      <c r="C473" t="n">
+        <v>1</v>
+      </c>
+      <c r="D473" t="n">
+        <v>15</v>
+      </c>
+      <c r="E473" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Breaks a
+  person's concentration</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>INTERRUPTION</t>
+        </is>
+      </c>
+      <c r="C474" t="n">
+        <v>1</v>
+      </c>
+      <c r="D474" t="n">
+        <v>15</v>
+      </c>
+      <c r="E474" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Focus
+  attention</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>CONCENTRATE</t>
+        </is>
+      </c>
+      <c r="C475" t="n">
+        <v>1</v>
+      </c>
+      <c r="D475" t="n">
+        <v>15</v>
+      </c>
+      <c r="E475" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Put the
+  most important demand first</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>PRIORITIZE</t>
+        </is>
+      </c>
+      <c r="C476" t="n">
+        <v>1</v>
+      </c>
+      <c r="D476" t="n">
+        <v>15</v>
+      </c>
+      <c r="E476" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>How
+  firmly a hand holds an object</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>GRIP</t>
+        </is>
+      </c>
+      <c r="C477" t="n">
+        <v>1</v>
+      </c>
+      <c r="D477" t="n">
+        <v>16</v>
+      </c>
+      <c r="E477" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Extend
+  an arm toward an object</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>REACH</t>
+        </is>
+      </c>
+      <c r="C478" t="n">
+        <v>1</v>
+      </c>
+      <c r="D478" t="n">
+        <v>16</v>
+      </c>
+      <c r="E478" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Joint
+  between the forearm and the hand</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>WRIST</t>
+        </is>
+      </c>
+      <c r="C479" t="n">
+        <v>3</v>
+      </c>
+      <c r="D479" t="n">
+        <v>16</v>
+      </c>
+      <c r="E479" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Ability
+  developed through learning and repeated use</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>SKILL</t>
+        </is>
+      </c>
+      <c r="C480" t="n">
+        <v>1</v>
+      </c>
+      <c r="D480" t="n">
+        <v>16</v>
+      </c>
+      <c r="E480" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Familiar
+  routine that may need little step-by-step thought</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>HABIT</t>
+        </is>
+      </c>
+      <c r="C481" t="n">
+        <v>2</v>
+      </c>
+      <c r="D481" t="n">
+        <v>16</v>
+      </c>
+      <c r="E481" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Close
+  the hand around an object to hold it</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>GRASP</t>
+        </is>
+      </c>
+      <c r="C482" t="n">
+        <v>2</v>
+      </c>
+      <c r="D482" t="n">
+        <v>16</v>
+      </c>
+      <c r="E482" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Body
+  tissue that contracts to move a joint</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>MUSCLE</t>
+        </is>
+      </c>
+      <c r="C483" t="n">
+        <v>3</v>
+      </c>
+      <c r="D483" t="n">
+        <v>16</v>
+      </c>
+      <c r="E483" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Let go
+  of something after holding it</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>RELEASE</t>
+        </is>
+      </c>
+      <c r="C484" t="n">
+        <v>2</v>
+      </c>
+      <c r="D484" t="n">
+        <v>16</v>
+      </c>
+      <c r="E484" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>How the
+  body is positioned during an activity</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>POSTURE</t>
+        </is>
+      </c>
+      <c r="C485" t="n">
+        <v>3</v>
+      </c>
+      <c r="D485" t="n">
+        <v>16</v>
+      </c>
+      <c r="E485" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Work on
+  improving an existing movement through guided practice</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>RETRAIN</t>
+        </is>
+      </c>
+      <c r="C486" t="n">
+        <v>1</v>
+      </c>
+      <c r="D486" t="n">
+        <v>16</v>
+      </c>
+      <c r="E486" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Smooth,
+  connected performance of a familiar action</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>FLUENCY</t>
+        </is>
+      </c>
+      <c r="C487" t="n">
+        <v>1</v>
+      </c>
+      <c r="D487" t="n">
+        <v>16</v>
+      </c>
+      <c r="E487" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Ordered
+  series of actions making up a learned skill</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>SEQUENCE</t>
+        </is>
+      </c>
+      <c r="C488" t="n">
+        <v>1</v>
+      </c>
+      <c r="D488" t="n">
+        <v>16</v>
+      </c>
+      <c r="E488" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Everyday
+  activity of putting on clothes</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>DRESSING</t>
+        </is>
+      </c>
+      <c r="C489" t="n">
+        <v>1</v>
+      </c>
+      <c r="D489" t="n">
+        <v>16</v>
+      </c>
+      <c r="E489" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Move
+  from one surface to another, such as bed to chair</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>TRANSFER</t>
+        </is>
+      </c>
+      <c r="C490" t="n">
+        <v>1</v>
+      </c>
+      <c r="D490" t="n">
+        <v>16</v>
+      </c>
+      <c r="E490" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Joint
+  connecting the upper arm to the body</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>SHOULDER</t>
+        </is>
+      </c>
+      <c r="C491" t="n">
+        <v>3</v>
+      </c>
+      <c r="D491" t="n">
+        <v>16</v>
+      </c>
+      <c r="E491" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Practise
+  an action in preparation for using it</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>REHEARSE</t>
+        </is>
+      </c>
+      <c r="C492" t="n">
+        <v>2</v>
+      </c>
+      <c r="D492" t="n">
+        <v>16</v>
+      </c>
+      <c r="E492" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Type of
+  memory for events a person has experienced</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>EPISODIC</t>
+        </is>
+      </c>
+      <c r="C493" t="n">
+        <v>3</v>
+      </c>
+      <c r="D493" t="n">
+        <v>16</v>
+      </c>
+      <c r="E493" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Describes
+  an intentional effort to move on command</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>VOLUNTARY</t>
+        </is>
+      </c>
+      <c r="C494" t="n">
+        <v>1</v>
+      </c>
+      <c r="D494" t="n">
+        <v>16</v>
+      </c>
+      <c r="E494" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Ability
+  to keep an activity going over time</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>ENDURANCE</t>
+        </is>
+      </c>
+      <c r="C495" t="n">
+        <v>1</v>
+      </c>
+      <c r="D495" t="n">
+        <v>16</v>
+      </c>
+      <c r="E495" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Help
+  that may still be needed even when some movement occurs</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>ASSISTANCE</t>
+        </is>
+      </c>
+      <c r="C496" t="n">
+        <v>1</v>
+      </c>
+      <c r="D496" t="n">
+        <v>16</v>
+      </c>
+      <c r="E496" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Brain
+  structure involved in fine-tuning movement and motor learning</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>CEREBELLUM</t>
+        </is>
+      </c>
+      <c r="C497" t="n">
+        <v>2</v>
+      </c>
+      <c r="D497" t="n">
+        <v>16</v>
+      </c>
+      <c r="E497" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Type of
+  memory that supports learned skills such as typing</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>PROCEDURAL</t>
+        </is>
+      </c>
+      <c r="C498" t="n">
+        <v>1</v>
+      </c>
+      <c r="D498" t="n">
+        <v>16</v>
+      </c>
+      <c r="E498" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Make
+  several muscles or joints work together on an action</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>COORDINATE</t>
+        </is>
+      </c>
+      <c r="C499" t="n">
+        <v>1</v>
+      </c>
+      <c r="D499" t="n">
+        <v>16</v>
+      </c>
+      <c r="E499" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Describes
+  an action that can be performed again in similar conditions</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>REPEATABLE</t>
+        </is>
+      </c>
+      <c r="C500" t="n">
+        <v>1</v>
+      </c>
+      <c r="D500" t="n">
+        <v>16</v>
+      </c>
+      <c r="E500" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Toward a
+  chosen target</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>AIM</t>
+        </is>
+      </c>
+      <c r="C501" t="n">
+        <v>1</v>
+      </c>
+      <c r="D501" t="n">
+        <v>17</v>
+      </c>
+      <c r="E501" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Can
+  provide movement timing</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>BEAT</t>
+        </is>
+      </c>
+      <c r="C502" t="n">
+        <v>3</v>
+      </c>
+      <c r="D502" t="n">
+        <v>17</v>
+      </c>
+      <c r="E502" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Store
+  your books here.</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>SHELF</t>
+        </is>
+      </c>
+      <c r="C503" t="n">
+        <v>3</v>
+      </c>
+      <c r="D503" t="n">
+        <v>17</v>
+      </c>
+      <c r="E503" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Firmly
+  in the hand.</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
+      <c r="C504" t="n">
+        <v>3</v>
+      </c>
+      <c r="D504" t="n">
+        <v>17</v>
+      </c>
+      <c r="E504" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Put an
+  object where it belongs</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>PLACE</t>
+        </is>
+      </c>
+      <c r="C505" t="n">
+        <v>3</v>
+      </c>
+      <c r="D505" t="n">
+        <v>17</v>
+      </c>
+      <c r="E505" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Physical
+  item whose shape and weight affect how it is handled</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>OBJECT</t>
+        </is>
+      </c>
+      <c r="C506" t="n">
+        <v>3</v>
+      </c>
+      <c r="D506" t="n">
+        <v>17</v>
+      </c>
+      <c r="E506" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>How
+  heavy an object is</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>WEIGHT</t>
+        </is>
+      </c>
+      <c r="C507" t="n">
+        <v>1</v>
+      </c>
+      <c r="D507" t="n">
+        <v>17</v>
+      </c>
+      <c r="E507" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Force
+  that makes lifting different from sliding on a table</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>GRAVITY</t>
+        </is>
+      </c>
+      <c r="C508" t="n">
+        <v>1</v>
+      </c>
+      <c r="D508" t="n">
+        <v>17</v>
+      </c>
+      <c r="E508" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Task,
+  surroundings and available help around an activity</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>CONTEXT</t>
+        </is>
+      </c>
+      <c r="C509" t="n">
+        <v>1</v>
+      </c>
+      <c r="D509" t="n">
+        <v>17</v>
+      </c>
+      <c r="E509" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>This
+  matters alongside task completion</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>COMFORT</t>
+        </is>
+      </c>
+      <c r="C510" t="n">
+        <v>2</v>
+      </c>
+      <c r="D510" t="n">
+        <v>17</v>
+      </c>
+      <c r="E510" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Doing
+  two things at once</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>DUALTASK</t>
+        </is>
+      </c>
+      <c r="C511" t="n">
+        <v>1</v>
+      </c>
+      <c r="D511" t="n">
+        <v>17</v>
+      </c>
+      <c r="E511" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Ffocus
+  directed toward a movement's destination.</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>EXTERNAL</t>
+        </is>
+      </c>
+      <c r="C512" t="n">
+        <v>1</v>
+      </c>
+      <c r="D512" t="n">
+        <v>17</v>
+      </c>
+      <c r="E512" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Focus
+  directed toward the body's own movements</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>INTERNAL</t>
+        </is>
+      </c>
+      <c r="C513" t="n">
+        <v>1</v>
+      </c>
+      <c r="D513" t="n">
+        <v>17</v>
+      </c>
+      <c r="E513" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Information
+  about how an activity went</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>FEEDBACK</t>
+        </is>
+      </c>
+      <c r="C514" t="n">
+        <v>1</v>
+      </c>
+      <c r="D514" t="n">
+        <v>17</v>
+      </c>
+      <c r="E514" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Using a
+  helpful strategy outside the setting where it was learned</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>CARRYOVER</t>
+        </is>
+      </c>
+      <c r="C515" t="n">
+        <v>1</v>
+      </c>
+      <c r="D515" t="n">
+        <v>17</v>
+      </c>
+      <c r="E515" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Move
+  items around to make a task easier</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>REARRANGE</t>
+        </is>
+      </c>
+      <c r="C516" t="n">
+        <v>1</v>
+      </c>
+      <c r="D516" t="n">
+        <v>17</v>
+      </c>
+      <c r="E516" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Qualified
+  professional who can help choose suitable rehabilitation tasks</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>THERAPIST</t>
+        </is>
+      </c>
+      <c r="C517" t="n">
+        <v>3</v>
+      </c>
+      <c r="D517" t="n">
+        <v>17</v>
+      </c>
+      <c r="E517" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>A person
+  whose preferences and responses may differ from others</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>INDIVIDUAL</t>
+        </is>
+      </c>
+      <c r="C518" t="n">
+        <v>2</v>
+      </c>
+      <c r="D518" t="n">
+        <v>17</v>
+      </c>
+      <c r="E518" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Description
+  of what someone noticed</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>OBSERVATION</t>
+        </is>
+      </c>
+      <c r="C519" t="n">
+        <v>1</v>
+      </c>
+      <c r="D519" t="n">
+        <v>17</v>
+      </c>
+      <c r="E519" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>